<commit_message>
feat: install the QoL build into the game
install the QoL build into the game; item amounts, glossary and % fixes

From the project's review of the game screen: - build_variant.py now
installs a verified build into the game folder (install_variant.py): the
variant's files plus the untouched originals, nothing else; replaced
files are saved in build/installed_backup/. - Items: the exact amount
replaces the vague size, never both ("Restore an ally's HP (+250)."),
checked against the binary. - Enchant names: figures from the first
game's guide are shown too (142 names), resistance is written with %,
and names keep the game's own words (Enmity, resistance). - Skill boxes:
resistance with %. Line 1 stays vanilla, so the battle bar carries no
level-dependent figure.

55 tests.
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/qol_enchant_text.xlsx
+++ b/mod_project/data_tables/qol_enchant_text.xlsx
@@ -669,21 +669,17 @@
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Max HP DOWN</t>
+          <t>Max HP -10%</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
-      <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="2" t="inlineStr">
-        <is>
-          <t>Max HP -10%</t>
-        </is>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
+      <c r="I4" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
           <t>The DT2-2 wiki lists this one as unknown (-??%)</t>
@@ -2187,21 +2183,17 @@
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>Physical attack UP</t>
+          <t>Physical attack +4%</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr"/>
-      <c r="I31" s="2" t="inlineStr"/>
-      <c r="J31" s="2" t="inlineStr">
-        <is>
-          <t>Physical attack +4%</t>
-        </is>
-      </c>
-      <c r="K31" s="2" t="inlineStr">
+      <c r="I31" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr"/>
       <c r="L31" s="2" t="inlineStr">
         <is>
           <t>First game: stacks up to +50%</t>
@@ -2249,21 +2241,17 @@
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>Physical attack MiniUP</t>
+          <t>Physical attack +2%</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr"/>
-      <c r="I32" s="2" t="inlineStr"/>
-      <c r="J32" s="2" t="inlineStr">
-        <is>
-          <t>Physical attack +2%</t>
-        </is>
-      </c>
-      <c r="K32" s="2" t="inlineStr">
+      <c r="I32" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J32" s="2" t="inlineStr"/>
+      <c r="K32" s="2" t="inlineStr"/>
       <c r="L32" s="2" t="inlineStr">
         <is>
           <t>First game: stacks up to +50%</t>
@@ -2611,21 +2599,17 @@
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>Magic attack UP</t>
+          <t>Magic attack +4%</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr"/>
-      <c r="I39" s="2" t="inlineStr"/>
-      <c r="J39" s="2" t="inlineStr">
-        <is>
-          <t>Magic attack +4%</t>
-        </is>
-      </c>
-      <c r="K39" s="2" t="inlineStr">
+      <c r="I39" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J39" s="2" t="inlineStr"/>
+      <c r="K39" s="2" t="inlineStr"/>
       <c r="L39" s="2" t="inlineStr">
         <is>
           <t>First game: stacks up to +50%</t>
@@ -2673,21 +2657,17 @@
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>Magic attack MiniUP</t>
+          <t>Magic attack +2%</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr"/>
-      <c r="I40" s="2" t="inlineStr"/>
-      <c r="J40" s="2" t="inlineStr">
-        <is>
-          <t>Magic attack +2%</t>
-        </is>
-      </c>
-      <c r="K40" s="2" t="inlineStr">
+      <c r="I40" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J40" s="2" t="inlineStr"/>
+      <c r="K40" s="2" t="inlineStr"/>
       <c r="L40" s="2" t="inlineStr">
         <is>
           <t>First game: stacks up to +50%</t>
@@ -3235,21 +3215,17 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Enmity UP</t>
+          <t>Enmity +5%</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr"/>
-      <c r="I51" s="2" t="inlineStr"/>
-      <c r="J51" s="2" t="inlineStr">
-        <is>
-          <t>Enmity +5%</t>
-        </is>
-      </c>
-      <c r="K51" s="2" t="inlineStr">
+      <c r="I51" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J51" s="2" t="inlineStr"/>
+      <c r="K51" s="2" t="inlineStr"/>
       <c r="L51" s="2" t="inlineStr"/>
       <c r="M51" s="2" t="inlineStr">
         <is>
@@ -3293,21 +3269,17 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Enmity DOWN</t>
+          <t>Enmity -5%</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr"/>
-      <c r="I52" s="2" t="inlineStr"/>
-      <c r="J52" s="2" t="inlineStr">
-        <is>
-          <t>Enmity -5%</t>
-        </is>
-      </c>
-      <c r="K52" s="2" t="inlineStr">
+      <c r="I52" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J52" s="2" t="inlineStr"/>
+      <c r="K52" s="2" t="inlineStr"/>
       <c r="L52" s="2" t="inlineStr"/>
       <c r="M52" s="2" t="inlineStr">
         <is>
@@ -3351,21 +3323,17 @@
       </c>
       <c r="G53" s="2" t="inlineStr">
         <is>
-          <t>Speed UP</t>
+          <t>Speed +10%</t>
         </is>
       </c>
       <c r="H53" s="2" t="inlineStr"/>
-      <c r="I53" s="2" t="inlineStr"/>
-      <c r="J53" s="2" t="inlineStr">
-        <is>
-          <t>Speed +10%</t>
-        </is>
-      </c>
-      <c r="K53" s="2" t="inlineStr">
+      <c r="I53" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J53" s="2" t="inlineStr"/>
+      <c r="K53" s="2" t="inlineStr"/>
       <c r="L53" s="2" t="inlineStr">
         <is>
           <t>DT2-2 player test: only five of them count</t>
@@ -3413,21 +3381,17 @@
       </c>
       <c r="G54" s="2" t="inlineStr">
         <is>
-          <t>Speed MiniUP</t>
+          <t>Speed +5%</t>
         </is>
       </c>
       <c r="H54" s="2" t="inlineStr"/>
-      <c r="I54" s="2" t="inlineStr"/>
-      <c r="J54" s="2" t="inlineStr">
-        <is>
-          <t>Speed +5%</t>
-        </is>
-      </c>
-      <c r="K54" s="2" t="inlineStr">
+      <c r="I54" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J54" s="2" t="inlineStr"/>
+      <c r="K54" s="2" t="inlineStr"/>
       <c r="L54" s="2" t="inlineStr"/>
       <c r="M54" s="2" t="inlineStr">
         <is>
@@ -3521,21 +3485,17 @@
       </c>
       <c r="G56" s="2" t="inlineStr">
         <is>
-          <t>Chant speed UP</t>
+          <t>Chant speed +20%</t>
         </is>
       </c>
       <c r="H56" s="2" t="inlineStr"/>
-      <c r="I56" s="2" t="inlineStr"/>
-      <c r="J56" s="2" t="inlineStr">
-        <is>
-          <t>Chant speed +20%</t>
-        </is>
-      </c>
-      <c r="K56" s="2" t="inlineStr">
+      <c r="I56" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J56" s="2" t="inlineStr"/>
+      <c r="K56" s="2" t="inlineStr"/>
       <c r="L56" s="2" t="inlineStr">
         <is>
           <t>DT2-2 player test: only three of them count</t>
@@ -3583,21 +3543,17 @@
       </c>
       <c r="G57" s="2" t="inlineStr">
         <is>
-          <t>Chant speed MiniUP</t>
+          <t>Chant speed +10%</t>
         </is>
       </c>
       <c r="H57" s="2" t="inlineStr"/>
-      <c r="I57" s="2" t="inlineStr"/>
-      <c r="J57" s="2" t="inlineStr">
-        <is>
-          <t>Chant speed +10%</t>
-        </is>
-      </c>
-      <c r="K57" s="2" t="inlineStr">
+      <c r="I57" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J57" s="2" t="inlineStr"/>
+      <c r="K57" s="2" t="inlineStr"/>
       <c r="L57" s="2" t="inlineStr"/>
       <c r="M57" s="2" t="inlineStr">
         <is>
@@ -3741,21 +3697,17 @@
       </c>
       <c r="G60" s="2" t="inlineStr">
         <is>
-          <t>Interruption rate DOWN</t>
+          <t>Interruption rate -6%</t>
         </is>
       </c>
       <c r="H60" s="2" t="inlineStr"/>
-      <c r="I60" s="2" t="inlineStr"/>
-      <c r="J60" s="2" t="inlineStr">
-        <is>
-          <t>Interruption rate -6%</t>
-        </is>
-      </c>
-      <c r="K60" s="2" t="inlineStr">
+      <c r="I60" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J60" s="2" t="inlineStr"/>
+      <c r="K60" s="2" t="inlineStr"/>
       <c r="L60" s="2" t="inlineStr"/>
       <c r="M60" s="2" t="inlineStr">
         <is>
@@ -3799,21 +3751,17 @@
       </c>
       <c r="G61" s="2" t="inlineStr">
         <is>
-          <t>Interruption rate MiniDOWN</t>
+          <t>Interruption rate -3%</t>
         </is>
       </c>
       <c r="H61" s="2" t="inlineStr"/>
-      <c r="I61" s="2" t="inlineStr"/>
-      <c r="J61" s="2" t="inlineStr">
-        <is>
-          <t>Interruption rate -3%</t>
-        </is>
-      </c>
-      <c r="K61" s="2" t="inlineStr">
+      <c r="I61" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J61" s="2" t="inlineStr"/>
+      <c r="K61" s="2" t="inlineStr"/>
       <c r="L61" s="2" t="inlineStr"/>
       <c r="M61" s="2" t="inlineStr">
         <is>
@@ -3857,21 +3805,17 @@
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Interruption rate UP</t>
+          <t>Interruption rate +6%</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr"/>
-      <c r="I62" s="2" t="inlineStr"/>
-      <c r="J62" s="2" t="inlineStr">
-        <is>
-          <t>Interruption rate +6%</t>
-        </is>
-      </c>
-      <c r="K62" s="2" t="inlineStr">
+      <c r="I62" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J62" s="2" t="inlineStr"/>
+      <c r="K62" s="2" t="inlineStr"/>
       <c r="L62" s="2" t="inlineStr"/>
       <c r="M62" s="2" t="inlineStr">
         <is>
@@ -4313,21 +4257,17 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Convert received damage into TP</t>
+          <t>Convert 5% of received damage into TP</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr"/>
-      <c r="I70" s="2" t="inlineStr"/>
-      <c r="J70" s="2" t="inlineStr">
-        <is>
-          <t>Convert 5% of received damage into TP</t>
-        </is>
-      </c>
-      <c r="K70" s="2" t="inlineStr">
+      <c r="I70" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J70" s="2" t="inlineStr"/>
+      <c r="K70" s="2" t="inlineStr"/>
       <c r="L70" s="2" t="inlineStr">
         <is>
           <t>First game: at least 1 TP, also from poison and traps</t>
@@ -4425,21 +4365,17 @@
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>Fire magic buff</t>
+          <t>Fire magic +20%</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr"/>
-      <c r="I72" s="2" t="inlineStr"/>
-      <c r="J72" s="2" t="inlineStr">
-        <is>
-          <t>Fire magic +20%</t>
-        </is>
-      </c>
-      <c r="K72" s="2" t="inlineStr">
+      <c r="I72" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J72" s="2" t="inlineStr"/>
+      <c r="K72" s="2" t="inlineStr"/>
       <c r="L72" s="2" t="inlineStr">
         <is>
           <t>First game: magic of that element x1.2, and the weapon attacks with that element</t>
@@ -4487,21 +4423,17 @@
       </c>
       <c r="G73" s="2" t="inlineStr">
         <is>
-          <t>Water magic buff</t>
+          <t>Water magic +20%</t>
         </is>
       </c>
       <c r="H73" s="2" t="inlineStr"/>
-      <c r="I73" s="2" t="inlineStr"/>
-      <c r="J73" s="2" t="inlineStr">
-        <is>
-          <t>Water magic +20%</t>
-        </is>
-      </c>
-      <c r="K73" s="2" t="inlineStr">
+      <c r="I73" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J73" s="2" t="inlineStr"/>
+      <c r="K73" s="2" t="inlineStr"/>
       <c r="L73" s="2" t="inlineStr">
         <is>
           <t>First game: magic of that element x1.2, and the weapon attacks with that element</t>
@@ -4549,21 +4481,17 @@
       </c>
       <c r="G74" s="2" t="inlineStr">
         <is>
-          <t>Wind magic buff</t>
+          <t>Wind magic +20%</t>
         </is>
       </c>
       <c r="H74" s="2" t="inlineStr"/>
-      <c r="I74" s="2" t="inlineStr"/>
-      <c r="J74" s="2" t="inlineStr">
-        <is>
-          <t>Wind magic +20%</t>
-        </is>
-      </c>
-      <c r="K74" s="2" t="inlineStr">
+      <c r="I74" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J74" s="2" t="inlineStr"/>
+      <c r="K74" s="2" t="inlineStr"/>
       <c r="L74" s="2" t="inlineStr">
         <is>
           <t>First game: magic of that element x1.2, and the weapon attacks with that element</t>
@@ -4611,21 +4539,17 @@
       </c>
       <c r="G75" s="2" t="inlineStr">
         <is>
-          <t>Earth magic buff</t>
+          <t>Earth magic +20%</t>
         </is>
       </c>
       <c r="H75" s="2" t="inlineStr"/>
-      <c r="I75" s="2" t="inlineStr"/>
-      <c r="J75" s="2" t="inlineStr">
-        <is>
-          <t>Earth magic +20%</t>
-        </is>
-      </c>
-      <c r="K75" s="2" t="inlineStr">
+      <c r="I75" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J75" s="2" t="inlineStr"/>
+      <c r="K75" s="2" t="inlineStr"/>
       <c r="L75" s="2" t="inlineStr">
         <is>
           <t>First game: magic of that element x1.2, and the weapon attacks with that element</t>
@@ -4673,21 +4597,17 @@
       </c>
       <c r="G76" s="2" t="inlineStr">
         <is>
-          <t>Lightning magic buff</t>
+          <t>Lightning magic +20%</t>
         </is>
       </c>
       <c r="H76" s="2" t="inlineStr"/>
-      <c r="I76" s="2" t="inlineStr"/>
-      <c r="J76" s="2" t="inlineStr">
-        <is>
-          <t>Lightning magic +20%</t>
-        </is>
-      </c>
-      <c r="K76" s="2" t="inlineStr">
+      <c r="I76" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J76" s="2" t="inlineStr"/>
+      <c r="K76" s="2" t="inlineStr"/>
       <c r="L76" s="2" t="inlineStr">
         <is>
           <t>First game: magic of that element x1.2, and the weapon attacks with that element</t>
@@ -4735,7 +4655,7 @@
       </c>
       <c r="G77" s="2" t="inlineStr">
         <is>
-          <t>Fire resistance +20</t>
+          <t>Fire resistance +20%</t>
         </is>
       </c>
       <c r="H77" s="2" t="inlineStr"/>
@@ -4789,7 +4709,7 @@
       </c>
       <c r="G78" s="2" t="inlineStr">
         <is>
-          <t>Fire resistance +10</t>
+          <t>Fire resistance +10%</t>
         </is>
       </c>
       <c r="H78" s="2" t="inlineStr"/>
@@ -4843,7 +4763,7 @@
       </c>
       <c r="G79" s="2" t="inlineStr">
         <is>
-          <t>Fire resistance -20</t>
+          <t>Fire resistance -20%</t>
         </is>
       </c>
       <c r="H79" s="2" t="inlineStr"/>
@@ -4897,7 +4817,7 @@
       </c>
       <c r="G80" s="2" t="inlineStr">
         <is>
-          <t>Water resistance +20</t>
+          <t>Water resistance +20%</t>
         </is>
       </c>
       <c r="H80" s="2" t="inlineStr"/>
@@ -4951,7 +4871,7 @@
       </c>
       <c r="G81" s="2" t="inlineStr">
         <is>
-          <t>Water resistance +10</t>
+          <t>Water resistance +10%</t>
         </is>
       </c>
       <c r="H81" s="2" t="inlineStr"/>
@@ -5005,7 +4925,7 @@
       </c>
       <c r="G82" s="2" t="inlineStr">
         <is>
-          <t>Water resistance -20</t>
+          <t>Water resistance -20%</t>
         </is>
       </c>
       <c r="H82" s="2" t="inlineStr"/>
@@ -5059,7 +4979,7 @@
       </c>
       <c r="G83" s="2" t="inlineStr">
         <is>
-          <t>Wind resistance +20</t>
+          <t>Wind resistance +20%</t>
         </is>
       </c>
       <c r="H83" s="2" t="inlineStr"/>
@@ -5113,7 +5033,7 @@
       </c>
       <c r="G84" s="2" t="inlineStr">
         <is>
-          <t>Wind resistance +10</t>
+          <t>Wind resistance +10%</t>
         </is>
       </c>
       <c r="H84" s="2" t="inlineStr"/>
@@ -5167,7 +5087,7 @@
       </c>
       <c r="G85" s="2" t="inlineStr">
         <is>
-          <t>Wind resistance -20</t>
+          <t>Wind resistance -20%</t>
         </is>
       </c>
       <c r="H85" s="2" t="inlineStr"/>
@@ -5221,7 +5141,7 @@
       </c>
       <c r="G86" s="2" t="inlineStr">
         <is>
-          <t>Earth resistance +20</t>
+          <t>Earth resistance +20%</t>
         </is>
       </c>
       <c r="H86" s="2" t="inlineStr"/>
@@ -5275,7 +5195,7 @@
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>Earth resistance +10</t>
+          <t>Earth resistance +10%</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr"/>
@@ -5329,7 +5249,7 @@
       </c>
       <c r="G88" s="2" t="inlineStr">
         <is>
-          <t>Earth resistance -20</t>
+          <t>Earth resistance -20%</t>
         </is>
       </c>
       <c r="H88" s="2" t="inlineStr"/>
@@ -5383,7 +5303,7 @@
       </c>
       <c r="G89" s="2" t="inlineStr">
         <is>
-          <t>Lightning resistance +20</t>
+          <t>Lightning resistance +20%</t>
         </is>
       </c>
       <c r="H89" s="2" t="inlineStr"/>
@@ -5437,7 +5357,7 @@
       </c>
       <c r="G90" s="2" t="inlineStr">
         <is>
-          <t>Lightning resistance +10</t>
+          <t>Lightning resistance +10%</t>
         </is>
       </c>
       <c r="H90" s="2" t="inlineStr"/>
@@ -5491,7 +5411,7 @@
       </c>
       <c r="G91" s="2" t="inlineStr">
         <is>
-          <t>Lightning resistance -20</t>
+          <t>Lightning resistance -20%</t>
         </is>
       </c>
       <c r="H91" s="2" t="inlineStr"/>
@@ -5541,7 +5461,7 @@
       <c r="F92" s="2" t="inlineStr"/>
       <c r="G92" s="2" t="inlineStr">
         <is>
-          <t>Elemental resistance +50</t>
+          <t>Elemental resistance +50%</t>
         </is>
       </c>
       <c r="H92" s="2" t="inlineStr"/>
@@ -5599,7 +5519,7 @@
       </c>
       <c r="G93" s="2" t="inlineStr">
         <is>
-          <t>Elemental resistance +15</t>
+          <t>Elemental resistance +15%</t>
         </is>
       </c>
       <c r="H93" s="2" t="inlineStr"/>
@@ -5657,7 +5577,7 @@
       </c>
       <c r="G94" s="2" t="inlineStr">
         <is>
-          <t>Elemental resistance +7</t>
+          <t>Elemental resistance +7%</t>
         </is>
       </c>
       <c r="H94" s="2" t="inlineStr"/>
@@ -5715,7 +5635,7 @@
       </c>
       <c r="G95" s="2" t="inlineStr">
         <is>
-          <t>Elemental resistance -15</t>
+          <t>Elemental resistance -15%</t>
         </is>
       </c>
       <c r="H95" s="2" t="inlineStr"/>
@@ -5773,7 +5693,7 @@
       </c>
       <c r="G96" s="2" t="inlineStr">
         <is>
-          <t>Slash resistance +20</t>
+          <t>Slash resistance +20%</t>
         </is>
       </c>
       <c r="H96" s="2" t="inlineStr"/>
@@ -5827,7 +5747,7 @@
       </c>
       <c r="G97" s="2" t="inlineStr">
         <is>
-          <t>Slash resistance +10</t>
+          <t>Slash resistance +10%</t>
         </is>
       </c>
       <c r="H97" s="2" t="inlineStr"/>
@@ -5881,7 +5801,7 @@
       </c>
       <c r="G98" s="2" t="inlineStr">
         <is>
-          <t>Slash resistance -20</t>
+          <t>Slash resistance -20%</t>
         </is>
       </c>
       <c r="H98" s="2" t="inlineStr"/>
@@ -5935,7 +5855,7 @@
       </c>
       <c r="G99" s="2" t="inlineStr">
         <is>
-          <t>Stab resistance +20</t>
+          <t>Stab resistance +20%</t>
         </is>
       </c>
       <c r="H99" s="2" t="inlineStr"/>
@@ -5989,7 +5909,7 @@
       </c>
       <c r="G100" s="2" t="inlineStr">
         <is>
-          <t>Stab resistance +10</t>
+          <t>Stab resistance +10%</t>
         </is>
       </c>
       <c r="H100" s="2" t="inlineStr"/>
@@ -6043,7 +5963,7 @@
       </c>
       <c r="G101" s="2" t="inlineStr">
         <is>
-          <t>Stab resistance -20</t>
+          <t>Stab resistance -20%</t>
         </is>
       </c>
       <c r="H101" s="2" t="inlineStr"/>
@@ -6097,7 +6017,7 @@
       </c>
       <c r="G102" s="2" t="inlineStr">
         <is>
-          <t>Bash resistance +20</t>
+          <t>Bash resistance +20%</t>
         </is>
       </c>
       <c r="H102" s="2" t="inlineStr"/>
@@ -6151,7 +6071,7 @@
       </c>
       <c r="G103" s="2" t="inlineStr">
         <is>
-          <t>Bash resistance +10</t>
+          <t>Bash resistance +10%</t>
         </is>
       </c>
       <c r="H103" s="2" t="inlineStr"/>
@@ -6205,7 +6125,7 @@
       </c>
       <c r="G104" s="2" t="inlineStr">
         <is>
-          <t>Bash resistance -20</t>
+          <t>Bash resistance -20%</t>
         </is>
       </c>
       <c r="H104" s="2" t="inlineStr"/>
@@ -6255,7 +6175,7 @@
       <c r="F105" s="2" t="inlineStr"/>
       <c r="G105" s="2" t="inlineStr">
         <is>
-          <t>Physical resistance +25</t>
+          <t>Physical resistance +25%</t>
         </is>
       </c>
       <c r="H105" s="2" t="inlineStr"/>
@@ -6278,7 +6198,7 @@
       </c>
       <c r="N105" s="2" t="inlineStr">
         <is>
-          <t>contradicts dt22-wiki (Physical resistance +25)</t>
+          <t>contradicts dt22-wiki (Physical resistance +25%)</t>
         </is>
       </c>
     </row>
@@ -6313,7 +6233,7 @@
       </c>
       <c r="G106" s="2" t="inlineStr">
         <is>
-          <t>Physical resistance +10</t>
+          <t>Physical resistance +10%</t>
         </is>
       </c>
       <c r="H106" s="2" t="inlineStr"/>
@@ -6336,7 +6256,7 @@
       </c>
       <c r="N106" s="2" t="inlineStr">
         <is>
-          <t>contradicts dt22-wiki (Physical resistance +10)</t>
+          <t>contradicts dt22-wiki (Physical resistance +10%)</t>
         </is>
       </c>
     </row>
@@ -6371,7 +6291,7 @@
       </c>
       <c r="G107" s="2" t="inlineStr">
         <is>
-          <t>Physical resistance +5</t>
+          <t>Physical resistance +5%</t>
         </is>
       </c>
       <c r="H107" s="2" t="inlineStr"/>
@@ -6394,7 +6314,7 @@
       </c>
       <c r="N107" s="2" t="inlineStr">
         <is>
-          <t>contradicts dt22-wiki (Physical resistance +5)</t>
+          <t>contradicts dt22-wiki (Physical resistance +5%)</t>
         </is>
       </c>
     </row>
@@ -6429,21 +6349,17 @@
       </c>
       <c r="G108" s="2" t="inlineStr">
         <is>
-          <t>Physical resistance DOWN</t>
+          <t>Physical resistance -10%</t>
         </is>
       </c>
       <c r="H108" s="2" t="inlineStr"/>
-      <c r="I108" s="2" t="inlineStr"/>
-      <c r="J108" s="2" t="inlineStr">
-        <is>
-          <t>Physical resistance -10</t>
-        </is>
-      </c>
-      <c r="K108" s="2" t="inlineStr">
+      <c r="I108" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J108" s="2" t="inlineStr"/>
+      <c r="K108" s="2" t="inlineStr"/>
       <c r="L108" s="2" t="inlineStr">
         <is>
           <t>Slash, stab and bash. The DT2-2 wiki lists this one as unknown (-??)</t>
@@ -6456,7 +6372,7 @@
       </c>
       <c r="N108" s="2" t="inlineStr">
         <is>
-          <t>contradicts dt2-wiki (Physical resistance -10)</t>
+          <t>contradicts dt2-wiki (Physical resistance -10%)</t>
         </is>
       </c>
     </row>
@@ -8131,21 +8047,17 @@
       <c r="F143" s="2" t="inlineStr"/>
       <c r="G143" s="2" t="inlineStr">
         <is>
-          <t>Normal attacks absorb lots of HP</t>
+          <t>Normal attacks absorb HP (50% of damage)</t>
         </is>
       </c>
       <c r="H143" s="2" t="inlineStr"/>
-      <c r="I143" s="2" t="inlineStr"/>
-      <c r="J143" s="2" t="inlineStr">
-        <is>
-          <t>Normal attacks absorb 50% of damage as HP</t>
-        </is>
-      </c>
-      <c r="K143" s="2" t="inlineStr">
+      <c r="I143" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J143" s="2" t="inlineStr"/>
+      <c r="K143" s="2" t="inlineStr"/>
       <c r="L143" s="2" t="inlineStr">
         <is>
           <t>First game: no effect on undead</t>
@@ -8193,21 +8105,17 @@
       </c>
       <c r="G144" s="2" t="inlineStr">
         <is>
-          <t>Normal attacks absorb HP</t>
+          <t>Normal attacks absorb HP (15% of damage)</t>
         </is>
       </c>
       <c r="H144" s="2" t="inlineStr"/>
-      <c r="I144" s="2" t="inlineStr"/>
-      <c r="J144" s="2" t="inlineStr">
-        <is>
-          <t>Normal attacks absorb 15% of damage as HP</t>
-        </is>
-      </c>
-      <c r="K144" s="2" t="inlineStr">
+      <c r="I144" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J144" s="2" t="inlineStr"/>
+      <c r="K144" s="2" t="inlineStr"/>
       <c r="L144" s="2" t="inlineStr">
         <is>
           <t>First game: no effect on undead</t>
@@ -8220,7 +8128,7 @@
       </c>
       <c r="N144" s="2" t="inlineStr">
         <is>
-          <t>contradicts dt2-wiki (Normal attacks absorb 15% of damage as HP)</t>
+          <t>contradicts dt2-wiki (Normal attacks absorb HP (15% of damage))</t>
         </is>
       </c>
     </row>
@@ -8251,21 +8159,17 @@
       <c r="F145" s="2" t="inlineStr"/>
       <c r="G145" s="2" t="inlineStr">
         <is>
-          <t>Normal attacks absorb lots of TP</t>
+          <t>Normal attacks absorb TP (20% of damage)</t>
         </is>
       </c>
       <c r="H145" s="2" t="inlineStr"/>
-      <c r="I145" s="2" t="inlineStr"/>
-      <c r="J145" s="2" t="inlineStr">
-        <is>
-          <t>Normal attacks absorb 20% of damage as TP</t>
-        </is>
-      </c>
-      <c r="K145" s="2" t="inlineStr">
+      <c r="I145" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J145" s="2" t="inlineStr"/>
+      <c r="K145" s="2" t="inlineStr"/>
       <c r="L145" s="2" t="inlineStr">
         <is>
           <t>First game: no effect on undead</t>
@@ -8313,21 +8217,17 @@
       </c>
       <c r="G146" s="2" t="inlineStr">
         <is>
-          <t>Normal attacks absorb TP</t>
+          <t>Normal attacks absorb TP (5% of damage)</t>
         </is>
       </c>
       <c r="H146" s="2" t="inlineStr"/>
-      <c r="I146" s="2" t="inlineStr"/>
-      <c r="J146" s="2" t="inlineStr">
-        <is>
-          <t>Normal attacks absorb 5% of damage as TP</t>
-        </is>
-      </c>
-      <c r="K146" s="2" t="inlineStr">
+      <c r="I146" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J146" s="2" t="inlineStr"/>
+      <c r="K146" s="2" t="inlineStr"/>
       <c r="L146" s="2" t="inlineStr">
         <is>
           <t>First game: no effect on undead</t>
@@ -8340,7 +8240,7 @@
       </c>
       <c r="N146" s="2" t="inlineStr">
         <is>
-          <t>contradicts dt2-wiki (Normal attacks absorb 5% of damage as TP)</t>
+          <t>contradicts dt2-wiki (Normal attacks absorb TP (5% of damage))</t>
         </is>
       </c>
     </row>
@@ -8421,21 +8321,17 @@
       <c r="F148" s="2" t="inlineStr"/>
       <c r="G148" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Demons GrandUP</t>
+          <t>Physical attack vs. Demons +40%</t>
         </is>
       </c>
       <c r="H148" s="2" t="inlineStr"/>
-      <c r="I148" s="2" t="inlineStr"/>
-      <c r="J148" s="2" t="inlineStr">
-        <is>
-          <t>Physical attack vs. Demons +40%</t>
-        </is>
-      </c>
-      <c r="K148" s="2" t="inlineStr">
+      <c r="I148" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J148" s="2" t="inlineStr"/>
+      <c r="K148" s="2" t="inlineStr"/>
       <c r="L148" s="2" t="inlineStr">
         <is>
           <t>First game: physical damage x1.4</t>
@@ -8483,21 +8379,17 @@
       </c>
       <c r="G149" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Demons UP</t>
+          <t>Physical attack vs. Demons +20%</t>
         </is>
       </c>
       <c r="H149" s="2" t="inlineStr"/>
-      <c r="I149" s="2" t="inlineStr"/>
-      <c r="J149" s="2" t="inlineStr">
-        <is>
-          <t>Physical attack vs. Demons +20%</t>
-        </is>
-      </c>
-      <c r="K149" s="2" t="inlineStr">
+      <c r="I149" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J149" s="2" t="inlineStr"/>
+      <c r="K149" s="2" t="inlineStr"/>
       <c r="L149" s="2" t="inlineStr">
         <is>
           <t>First game: physical damage x1.2</t>
@@ -8541,21 +8433,17 @@
       <c r="F150" s="2" t="inlineStr"/>
       <c r="G150" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Apparitions GrandUP</t>
+          <t>Physical attack vs. Apparitions +40%</t>
         </is>
       </c>
       <c r="H150" s="2" t="inlineStr"/>
-      <c r="I150" s="2" t="inlineStr"/>
-      <c r="J150" s="2" t="inlineStr">
-        <is>
-          <t>Physical attack vs. Apparitions +40%</t>
-        </is>
-      </c>
-      <c r="K150" s="2" t="inlineStr">
+      <c r="I150" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J150" s="2" t="inlineStr"/>
+      <c r="K150" s="2" t="inlineStr"/>
       <c r="L150" s="2" t="inlineStr">
         <is>
           <t>First game: physical damage x1.4</t>
@@ -8603,21 +8491,17 @@
       </c>
       <c r="G151" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Apparitions UP</t>
+          <t>Physical attack vs. Apparitions +20%</t>
         </is>
       </c>
       <c r="H151" s="2" t="inlineStr"/>
-      <c r="I151" s="2" t="inlineStr"/>
-      <c r="J151" s="2" t="inlineStr">
-        <is>
-          <t>Physical attack vs. Apparitions +20%</t>
-        </is>
-      </c>
-      <c r="K151" s="2" t="inlineStr">
+      <c r="I151" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J151" s="2" t="inlineStr"/>
+      <c r="K151" s="2" t="inlineStr"/>
       <c r="L151" s="2" t="inlineStr">
         <is>
           <t>First game: physical damage x1.2</t>
@@ -8661,21 +8545,17 @@
       <c r="F152" s="2" t="inlineStr"/>
       <c r="G152" s="2" t="inlineStr">
         <is>
-          <t>Phys. attack vs. Magic Beings GrandUP</t>
+          <t>Phys. attack vs. Magic Beings +40%</t>
         </is>
       </c>
       <c r="H152" s="2" t="inlineStr"/>
-      <c r="I152" s="2" t="inlineStr"/>
-      <c r="J152" s="2" t="inlineStr">
-        <is>
-          <t>Phys. attack vs. Magic Beings +40%</t>
-        </is>
-      </c>
-      <c r="K152" s="2" t="inlineStr">
+      <c r="I152" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J152" s="2" t="inlineStr"/>
+      <c r="K152" s="2" t="inlineStr"/>
       <c r="L152" s="2" t="inlineStr">
         <is>
           <t>First game: physical damage x1.4</t>
@@ -8723,21 +8603,17 @@
       </c>
       <c r="G153" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Magic Beings UP</t>
+          <t>Physical attack vs. Magic Beings +20%</t>
         </is>
       </c>
       <c r="H153" s="2" t="inlineStr"/>
-      <c r="I153" s="2" t="inlineStr"/>
-      <c r="J153" s="2" t="inlineStr">
-        <is>
-          <t>Physical attack vs. Magic Beings +20%</t>
-        </is>
-      </c>
-      <c r="K153" s="2" t="inlineStr">
+      <c r="I153" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J153" s="2" t="inlineStr"/>
+      <c r="K153" s="2" t="inlineStr"/>
       <c r="L153" s="2" t="inlineStr">
         <is>
           <t>First game: physical damage x1.2</t>
@@ -8781,21 +8657,17 @@
       <c r="F154" s="2" t="inlineStr"/>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Humans MegaUP</t>
+          <t>Physical attack vs. Humans +100%</t>
         </is>
       </c>
       <c r="H154" s="2" t="inlineStr"/>
-      <c r="I154" s="2" t="inlineStr"/>
-      <c r="J154" s="2" t="inlineStr">
-        <is>
-          <t>Physical attack vs. Humans +100%</t>
-        </is>
-      </c>
-      <c r="K154" s="2" t="inlineStr">
+      <c r="I154" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J154" s="2" t="inlineStr"/>
+      <c r="K154" s="2" t="inlineStr"/>
       <c r="L154" s="2" t="inlineStr">
         <is>
           <t>First game: physical damage x2</t>
@@ -8839,21 +8711,17 @@
       <c r="F155" s="2" t="inlineStr"/>
       <c r="G155" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Humans GrandUP</t>
+          <t>Physical attack vs. Humans +40%</t>
         </is>
       </c>
       <c r="H155" s="2" t="inlineStr"/>
-      <c r="I155" s="2" t="inlineStr"/>
-      <c r="J155" s="2" t="inlineStr">
-        <is>
-          <t>Physical attack vs. Humans +40%</t>
-        </is>
-      </c>
-      <c r="K155" s="2" t="inlineStr">
+      <c r="I155" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J155" s="2" t="inlineStr"/>
+      <c r="K155" s="2" t="inlineStr"/>
       <c r="L155" s="2" t="inlineStr">
         <is>
           <t>First game: physical damage x1.4</t>
@@ -8901,21 +8769,17 @@
       </c>
       <c r="G156" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Humans UP</t>
+          <t>Physical attack vs. Humans +20%</t>
         </is>
       </c>
       <c r="H156" s="2" t="inlineStr"/>
-      <c r="I156" s="2" t="inlineStr"/>
-      <c r="J156" s="2" t="inlineStr">
-        <is>
-          <t>Physical attack vs. Humans +20%</t>
-        </is>
-      </c>
-      <c r="K156" s="2" t="inlineStr">
+      <c r="I156" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J156" s="2" t="inlineStr"/>
+      <c r="K156" s="2" t="inlineStr"/>
       <c r="L156" s="2" t="inlineStr">
         <is>
           <t>First game: physical damage x1.2</t>
@@ -8959,21 +8823,17 @@
       <c r="F157" s="2" t="inlineStr"/>
       <c r="G157" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Undead GrandUP</t>
+          <t>Physical attack vs. Undead +40%</t>
         </is>
       </c>
       <c r="H157" s="2" t="inlineStr"/>
-      <c r="I157" s="2" t="inlineStr"/>
-      <c r="J157" s="2" t="inlineStr">
-        <is>
-          <t>Physical attack vs. Undead +40%</t>
-        </is>
-      </c>
-      <c r="K157" s="2" t="inlineStr">
+      <c r="I157" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J157" s="2" t="inlineStr"/>
+      <c r="K157" s="2" t="inlineStr"/>
       <c r="L157" s="2" t="inlineStr">
         <is>
           <t>First game: physical damage x1.4</t>
@@ -9021,21 +8881,17 @@
       </c>
       <c r="G158" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Undead UP</t>
+          <t>Physical attack vs. Undead +20%</t>
         </is>
       </c>
       <c r="H158" s="2" t="inlineStr"/>
-      <c r="I158" s="2" t="inlineStr"/>
-      <c r="J158" s="2" t="inlineStr">
-        <is>
-          <t>Physical attack vs. Undead +20%</t>
-        </is>
-      </c>
-      <c r="K158" s="2" t="inlineStr">
+      <c r="I158" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J158" s="2" t="inlineStr"/>
+      <c r="K158" s="2" t="inlineStr"/>
       <c r="L158" s="2" t="inlineStr">
         <is>
           <t>First game: physical damage x1.2</t>
@@ -9079,21 +8935,17 @@
       <c r="F159" s="2" t="inlineStr"/>
       <c r="G159" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Dragons GrandUP</t>
+          <t>Physical attack vs. Dragons +40%</t>
         </is>
       </c>
       <c r="H159" s="2" t="inlineStr"/>
-      <c r="I159" s="2" t="inlineStr"/>
-      <c r="J159" s="2" t="inlineStr">
-        <is>
-          <t>Physical attack vs. Dragons +40%</t>
-        </is>
-      </c>
-      <c r="K159" s="2" t="inlineStr">
+      <c r="I159" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J159" s="2" t="inlineStr"/>
+      <c r="K159" s="2" t="inlineStr"/>
       <c r="L159" s="2" t="inlineStr">
         <is>
           <t>First game: physical damage x1.4</t>
@@ -9141,21 +8993,17 @@
       </c>
       <c r="G160" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Dragons UP</t>
+          <t>Physical attack vs. Dragons +20%</t>
         </is>
       </c>
       <c r="H160" s="2" t="inlineStr"/>
-      <c r="I160" s="2" t="inlineStr"/>
-      <c r="J160" s="2" t="inlineStr">
-        <is>
-          <t>Physical attack vs. Dragons +20%</t>
-        </is>
-      </c>
-      <c r="K160" s="2" t="inlineStr">
+      <c r="I160" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J160" s="2" t="inlineStr"/>
+      <c r="K160" s="2" t="inlineStr"/>
       <c r="L160" s="2" t="inlineStr">
         <is>
           <t>First game: physical damage x1.2</t>
@@ -9199,21 +9047,17 @@
       <c r="F161" s="2" t="inlineStr"/>
       <c r="G161" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Beasts GrandUP</t>
+          <t>Physical attack vs. Beasts +40%</t>
         </is>
       </c>
       <c r="H161" s="2" t="inlineStr"/>
-      <c r="I161" s="2" t="inlineStr"/>
-      <c r="J161" s="2" t="inlineStr">
-        <is>
-          <t>Physical attack vs. Beasts +40%</t>
-        </is>
-      </c>
-      <c r="K161" s="2" t="inlineStr">
+      <c r="I161" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J161" s="2" t="inlineStr"/>
+      <c r="K161" s="2" t="inlineStr"/>
       <c r="L161" s="2" t="inlineStr">
         <is>
           <t>First game: physical damage x1.4</t>
@@ -9261,21 +9105,17 @@
       </c>
       <c r="G162" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Beasts UP</t>
+          <t>Physical attack vs. Beasts +20%</t>
         </is>
       </c>
       <c r="H162" s="2" t="inlineStr"/>
-      <c r="I162" s="2" t="inlineStr"/>
-      <c r="J162" s="2" t="inlineStr">
-        <is>
-          <t>Physical attack vs. Beasts +20%</t>
-        </is>
-      </c>
-      <c r="K162" s="2" t="inlineStr">
+      <c r="I162" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J162" s="2" t="inlineStr"/>
+      <c r="K162" s="2" t="inlineStr"/>
       <c r="L162" s="2" t="inlineStr">
         <is>
           <t>First game: physical damage x1.2</t>
@@ -9319,21 +9159,17 @@
       <c r="F163" s="2" t="inlineStr"/>
       <c r="G163" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Fruit MegaUP</t>
+          <t>Physical attack vs. Fruit +100%</t>
         </is>
       </c>
       <c r="H163" s="2" t="inlineStr"/>
-      <c r="I163" s="2" t="inlineStr"/>
-      <c r="J163" s="2" t="inlineStr">
-        <is>
-          <t>Physical attack vs. Fruit +100%</t>
-        </is>
-      </c>
-      <c r="K163" s="2" t="inlineStr">
+      <c r="I163" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J163" s="2" t="inlineStr"/>
+      <c r="K163" s="2" t="inlineStr"/>
       <c r="L163" s="2" t="inlineStr">
         <is>
           <t>First game: physical damage x2</t>
@@ -9381,21 +9217,17 @@
       </c>
       <c r="G164" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Fruit GrandUP</t>
+          <t>Physical attack vs. Fruit +50%</t>
         </is>
       </c>
       <c r="H164" s="2" t="inlineStr"/>
-      <c r="I164" s="2" t="inlineStr"/>
-      <c r="J164" s="2" t="inlineStr">
-        <is>
-          <t>Physical attack vs. Fruit +50%</t>
-        </is>
-      </c>
-      <c r="K164" s="2" t="inlineStr">
+      <c r="I164" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J164" s="2" t="inlineStr"/>
+      <c r="K164" s="2" t="inlineStr"/>
       <c r="L164" s="2" t="inlineStr">
         <is>
           <t>First game: physical damage x1.5</t>
@@ -9623,21 +9455,17 @@
       <c r="F169" s="2" t="inlineStr"/>
       <c r="G169" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Felines MegaUP</t>
+          <t>Physical attack vs. Felines +100%</t>
         </is>
       </c>
       <c r="H169" s="2" t="inlineStr"/>
-      <c r="I169" s="2" t="inlineStr"/>
-      <c r="J169" s="2" t="inlineStr">
-        <is>
-          <t>Physical attack vs. Felines +100%</t>
-        </is>
-      </c>
-      <c r="K169" s="2" t="inlineStr">
+      <c r="I169" s="2" t="inlineStr">
         <is>
           <t>dt2-wiki</t>
         </is>
       </c>
+      <c r="J169" s="2" t="inlineStr"/>
+      <c r="K169" s="2" t="inlineStr"/>
       <c r="L169" s="2" t="inlineStr">
         <is>
           <t>First game: physical damage x2</t>
@@ -13609,7 +13437,7 @@
       <c r="F254" s="2" t="inlineStr"/>
       <c r="G254" s="2" t="inlineStr">
         <is>
-          <t>Fire resistance +100</t>
+          <t>Fire resistance +100%</t>
         </is>
       </c>
       <c r="H254" s="2" t="inlineStr"/>
@@ -13628,7 +13456,7 @@
       </c>
       <c r="N254" s="2" t="inlineStr">
         <is>
-          <t>contradicts dt22-wiki (Fire resistance +100)</t>
+          <t>contradicts dt22-wiki (Fire resistance +100%)</t>
         </is>
       </c>
     </row>
@@ -13659,7 +13487,7 @@
       <c r="F255" s="2" t="inlineStr"/>
       <c r="G255" s="2" t="inlineStr">
         <is>
-          <t>Fire resistance +50</t>
+          <t>Fire resistance +50%</t>
         </is>
       </c>
       <c r="H255" s="2" t="inlineStr"/>
@@ -13713,7 +13541,7 @@
       </c>
       <c r="G256" s="2" t="inlineStr">
         <is>
-          <t>Fire resistance -50</t>
+          <t>Fire resistance -50%</t>
         </is>
       </c>
       <c r="H256" s="2" t="inlineStr"/>
@@ -13732,7 +13560,7 @@
       </c>
       <c r="N256" s="2" t="inlineStr">
         <is>
-          <t>contradicts dt22-wiki (Fire resistance -50)</t>
+          <t>contradicts dt22-wiki (Fire resistance -50%)</t>
         </is>
       </c>
     </row>
@@ -13763,7 +13591,7 @@
       <c r="F257" s="2" t="inlineStr"/>
       <c r="G257" s="2" t="inlineStr">
         <is>
-          <t>Water resistance +100</t>
+          <t>Water resistance +100%</t>
         </is>
       </c>
       <c r="H257" s="2" t="inlineStr"/>
@@ -13782,7 +13610,7 @@
       </c>
       <c r="N257" s="2" t="inlineStr">
         <is>
-          <t>contradicts dt22-wiki (Water resistance +100)</t>
+          <t>contradicts dt22-wiki (Water resistance +100%)</t>
         </is>
       </c>
     </row>
@@ -13813,7 +13641,7 @@
       <c r="F258" s="2" t="inlineStr"/>
       <c r="G258" s="2" t="inlineStr">
         <is>
-          <t>Water resistance +50</t>
+          <t>Water resistance +50%</t>
         </is>
       </c>
       <c r="H258" s="2" t="inlineStr"/>
@@ -13867,7 +13695,7 @@
       </c>
       <c r="G259" s="2" t="inlineStr">
         <is>
-          <t>Water resistance -50</t>
+          <t>Water resistance -50%</t>
         </is>
       </c>
       <c r="H259" s="2" t="inlineStr"/>
@@ -13886,7 +13714,7 @@
       </c>
       <c r="N259" s="2" t="inlineStr">
         <is>
-          <t>contradicts dt22-wiki (Water resistance -50)</t>
+          <t>contradicts dt22-wiki (Water resistance -50%)</t>
         </is>
       </c>
     </row>
@@ -13917,7 +13745,7 @@
       <c r="F260" s="2" t="inlineStr"/>
       <c r="G260" s="2" t="inlineStr">
         <is>
-          <t>Wind resistance +100</t>
+          <t>Wind resistance +100%</t>
         </is>
       </c>
       <c r="H260" s="2" t="inlineStr"/>
@@ -13936,7 +13764,7 @@
       </c>
       <c r="N260" s="2" t="inlineStr">
         <is>
-          <t>contradicts dt22-wiki (Wind resistance +100)</t>
+          <t>contradicts dt22-wiki (Wind resistance +100%)</t>
         </is>
       </c>
     </row>
@@ -13967,7 +13795,7 @@
       <c r="F261" s="2" t="inlineStr"/>
       <c r="G261" s="2" t="inlineStr">
         <is>
-          <t>Wind resistance +50</t>
+          <t>Wind resistance +50%</t>
         </is>
       </c>
       <c r="H261" s="2" t="inlineStr"/>
@@ -14021,7 +13849,7 @@
       </c>
       <c r="G262" s="2" t="inlineStr">
         <is>
-          <t>Wind resistance -50</t>
+          <t>Wind resistance -50%</t>
         </is>
       </c>
       <c r="H262" s="2" t="inlineStr"/>
@@ -14040,7 +13868,7 @@
       </c>
       <c r="N262" s="2" t="inlineStr">
         <is>
-          <t>contradicts dt22-wiki (Wind resistance -50)</t>
+          <t>contradicts dt22-wiki (Wind resistance -50%)</t>
         </is>
       </c>
     </row>
@@ -14071,7 +13899,7 @@
       <c r="F263" s="2" t="inlineStr"/>
       <c r="G263" s="2" t="inlineStr">
         <is>
-          <t>Earth resistance +100</t>
+          <t>Earth resistance +100%</t>
         </is>
       </c>
       <c r="H263" s="2" t="inlineStr"/>
@@ -14090,7 +13918,7 @@
       </c>
       <c r="N263" s="2" t="inlineStr">
         <is>
-          <t>contradicts dt22-wiki (Earth resistance +100)</t>
+          <t>contradicts dt22-wiki (Earth resistance +100%)</t>
         </is>
       </c>
     </row>
@@ -14121,7 +13949,7 @@
       <c r="F264" s="2" t="inlineStr"/>
       <c r="G264" s="2" t="inlineStr">
         <is>
-          <t>Earth resistance +50</t>
+          <t>Earth resistance +50%</t>
         </is>
       </c>
       <c r="H264" s="2" t="inlineStr"/>
@@ -14175,7 +14003,7 @@
       </c>
       <c r="G265" s="2" t="inlineStr">
         <is>
-          <t>Earth resistance -50</t>
+          <t>Earth resistance -50%</t>
         </is>
       </c>
       <c r="H265" s="2" t="inlineStr"/>
@@ -14194,7 +14022,7 @@
       </c>
       <c r="N265" s="2" t="inlineStr">
         <is>
-          <t>contradicts dt22-wiki (Earth resistance -50)</t>
+          <t>contradicts dt22-wiki (Earth resistance -50%)</t>
         </is>
       </c>
     </row>
@@ -14225,7 +14053,7 @@
       <c r="F266" s="2" t="inlineStr"/>
       <c r="G266" s="2" t="inlineStr">
         <is>
-          <t>Lightning resistance +100</t>
+          <t>Lightning resistance +100%</t>
         </is>
       </c>
       <c r="H266" s="2" t="inlineStr"/>
@@ -14244,7 +14072,7 @@
       </c>
       <c r="N266" s="2" t="inlineStr">
         <is>
-          <t>contradicts dt22-wiki (Lightning resistance +100)</t>
+          <t>contradicts dt22-wiki (Lightning resistance +100%)</t>
         </is>
       </c>
     </row>
@@ -14275,7 +14103,7 @@
       <c r="F267" s="2" t="inlineStr"/>
       <c r="G267" s="2" t="inlineStr">
         <is>
-          <t>Lightning resistance +50</t>
+          <t>Lightning resistance +50%</t>
         </is>
       </c>
       <c r="H267" s="2" t="inlineStr"/>
@@ -14329,7 +14157,7 @@
       </c>
       <c r="G268" s="2" t="inlineStr">
         <is>
-          <t>Lightning resistance -50</t>
+          <t>Lightning resistance -50%</t>
         </is>
       </c>
       <c r="H268" s="2" t="inlineStr"/>
@@ -14348,7 +14176,7 @@
       </c>
       <c r="N268" s="2" t="inlineStr">
         <is>
-          <t>contradicts dt22-wiki (Lightning resistance -50)</t>
+          <t>contradicts dt22-wiki (Lightning resistance -50%)</t>
         </is>
       </c>
     </row>
@@ -14379,7 +14207,7 @@
       <c r="F269" s="2" t="inlineStr"/>
       <c r="G269" s="2" t="inlineStr">
         <is>
-          <t>Elemental resistance +75</t>
+          <t>Elemental resistance +75%</t>
         </is>
       </c>
       <c r="H269" s="2" t="inlineStr"/>
@@ -14402,7 +14230,7 @@
       </c>
       <c r="N269" s="2" t="inlineStr">
         <is>
-          <t>contradicts dt22-wiki (Elemental resistance +75)</t>
+          <t>contradicts dt22-wiki (Elemental resistance +75%)</t>
         </is>
       </c>
     </row>
@@ -14437,7 +14265,7 @@
       </c>
       <c r="G270" s="2" t="inlineStr">
         <is>
-          <t>Elemental resistance -30</t>
+          <t>Elemental resistance -30%</t>
         </is>
       </c>
       <c r="H270" s="2" t="inlineStr"/>
@@ -14491,7 +14319,7 @@
       <c r="F271" s="2" t="inlineStr"/>
       <c r="G271" s="2" t="inlineStr">
         <is>
-          <t>Slash resistance +100</t>
+          <t>Slash resistance +100%</t>
         </is>
       </c>
       <c r="H271" s="2" t="inlineStr"/>
@@ -14510,7 +14338,7 @@
       </c>
       <c r="N271" s="2" t="inlineStr">
         <is>
-          <t>contradicts dt22-wiki (Slash resistance +100)</t>
+          <t>contradicts dt22-wiki (Slash resistance +100%)</t>
         </is>
       </c>
     </row>
@@ -14541,7 +14369,7 @@
       <c r="F272" s="2" t="inlineStr"/>
       <c r="G272" s="2" t="inlineStr">
         <is>
-          <t>Slash resistance +50</t>
+          <t>Slash resistance +50%</t>
         </is>
       </c>
       <c r="H272" s="2" t="inlineStr"/>
@@ -14595,7 +14423,7 @@
       </c>
       <c r="G273" s="2" t="inlineStr">
         <is>
-          <t>Slash resistance -50</t>
+          <t>Slash resistance -50%</t>
         </is>
       </c>
       <c r="H273" s="2" t="inlineStr"/>
@@ -14614,7 +14442,7 @@
       </c>
       <c r="N273" s="2" t="inlineStr">
         <is>
-          <t>contradicts dt22-wiki (Slash resistance -50)</t>
+          <t>contradicts dt22-wiki (Slash resistance -50%)</t>
         </is>
       </c>
     </row>
@@ -14645,7 +14473,7 @@
       <c r="F274" s="2" t="inlineStr"/>
       <c r="G274" s="2" t="inlineStr">
         <is>
-          <t>Stab resistance +100</t>
+          <t>Stab resistance +100%</t>
         </is>
       </c>
       <c r="H274" s="2" t="inlineStr"/>
@@ -14664,7 +14492,7 @@
       </c>
       <c r="N274" s="2" t="inlineStr">
         <is>
-          <t>contradicts dt22-wiki (Stab resistance +100)</t>
+          <t>contradicts dt22-wiki (Stab resistance +100%)</t>
         </is>
       </c>
     </row>
@@ -14695,7 +14523,7 @@
       <c r="F275" s="2" t="inlineStr"/>
       <c r="G275" s="2" t="inlineStr">
         <is>
-          <t>Stab resistance +50</t>
+          <t>Stab resistance +50%</t>
         </is>
       </c>
       <c r="H275" s="2" t="inlineStr"/>
@@ -14749,7 +14577,7 @@
       </c>
       <c r="G276" s="2" t="inlineStr">
         <is>
-          <t>Stab resistance -50</t>
+          <t>Stab resistance -50%</t>
         </is>
       </c>
       <c r="H276" s="2" t="inlineStr"/>
@@ -14768,7 +14596,7 @@
       </c>
       <c r="N276" s="2" t="inlineStr">
         <is>
-          <t>contradicts dt22-wiki (Stab resistance -50)</t>
+          <t>contradicts dt22-wiki (Stab resistance -50%)</t>
         </is>
       </c>
     </row>
@@ -14799,7 +14627,7 @@
       <c r="F277" s="2" t="inlineStr"/>
       <c r="G277" s="2" t="inlineStr">
         <is>
-          <t>Bash resistance +100</t>
+          <t>Bash resistance +100%</t>
         </is>
       </c>
       <c r="H277" s="2" t="inlineStr"/>
@@ -14818,7 +14646,7 @@
       </c>
       <c r="N277" s="2" t="inlineStr">
         <is>
-          <t>contradicts dt22-wiki (Bash resistance +100)</t>
+          <t>contradicts dt22-wiki (Bash resistance +100%)</t>
         </is>
       </c>
     </row>
@@ -14849,7 +14677,7 @@
       <c r="F278" s="2" t="inlineStr"/>
       <c r="G278" s="2" t="inlineStr">
         <is>
-          <t>Bash resistance +50</t>
+          <t>Bash resistance +50%</t>
         </is>
       </c>
       <c r="H278" s="2" t="inlineStr"/>
@@ -14903,7 +14731,7 @@
       </c>
       <c r="G279" s="2" t="inlineStr">
         <is>
-          <t>Bash resistance -50</t>
+          <t>Bash resistance -50%</t>
         </is>
       </c>
       <c r="H279" s="2" t="inlineStr"/>
@@ -14922,7 +14750,7 @@
       </c>
       <c r="N279" s="2" t="inlineStr">
         <is>
-          <t>contradicts dt22-wiki (Bash resistance -50)</t>
+          <t>contradicts dt22-wiki (Bash resistance -50%)</t>
         </is>
       </c>
     </row>
@@ -14953,7 +14781,7 @@
       <c r="F280" s="2" t="inlineStr"/>
       <c r="G280" s="2" t="inlineStr">
         <is>
-          <t>Physical resistance +50</t>
+          <t>Physical resistance +50%</t>
         </is>
       </c>
       <c r="H280" s="2" t="inlineStr"/>
@@ -14976,7 +14804,7 @@
       </c>
       <c r="N280" s="2" t="inlineStr">
         <is>
-          <t>contradicts dt22-wiki (Physical resistance +50)</t>
+          <t>contradicts dt22-wiki (Physical resistance +50%)</t>
         </is>
       </c>
     </row>
@@ -15011,7 +14839,7 @@
       </c>
       <c r="G281" s="2" t="inlineStr">
         <is>
-          <t>Physical resistance -20</t>
+          <t>Physical resistance -20%</t>
         </is>
       </c>
       <c r="H281" s="2" t="inlineStr"/>
@@ -15034,7 +14862,7 @@
       </c>
       <c r="N281" s="2" t="inlineStr">
         <is>
-          <t>contradicts dt22-wiki (Physical resistance -20)</t>
+          <t>contradicts dt22-wiki (Physical resistance -20%)</t>
         </is>
       </c>
     </row>
@@ -15070,97 +14898,97 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>candidate from the first game only (vanilla name kept)</t>
+          <t>earlier build: agrees with dt2-wiki</t>
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>43</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>earlier build: agrees with dt2-wiki</t>
+          <t>earlier build: agrees with dt22-wiki</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>16</v>
+        <v>64</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>earlier build: agrees with dt22-wiki</t>
+          <t>earlier build: contradicts dt2-wiki</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>64</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>earlier build: contradicts dt2-wiki</t>
+          <t>earlier build: contradicts dt22-wiki</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>27</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>earlier build: contradicts dt22-wiki</t>
+          <t>earlier build: figure without a source</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>35</v>
+        <v>73</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>earlier build: figure without a source</t>
+          <t>earlier build: reworded, no new figure</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>73</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>earlier build: reworded, no new figure</t>
+          <t>earlier build: unchanged</t>
         </is>
       </c>
       <c r="B8" s="2" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>earlier build: unchanged</t>
+          <t>figure already in the vanilla name</t>
         </is>
       </c>
       <c r="B9" s="2" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>figure already in the vanilla name</t>
+          <t>figure from dt2-wiki</t>
         </is>
       </c>
       <c r="B10" s="2" t="n">
-        <v>37</v>
+        <v>43</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>figure from the guide of this game</t>
+          <t>figure from dt22-wiki</t>
         </is>
       </c>
       <c r="B11" s="2" t="n">
@@ -15236,12 +15064,12 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Japanese wiki of the first Dungeon Travelers 2, https://w.atwiki.jp/dungeon-travelers2/pages/200.html (same system, another game: candidate only)</t>
+          <t>Japanese wiki of the first Dungeon Travelers 2, https://w.atwiki.jp/dungeon-travelers2/pages/200.html (same system, another game: not confirmed for this one)</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>no</t>
+          <t>yes</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
qol: apply 102 verified enchantments from x86 binary reverse engineering
- Add 'exe-verified' source to qol_rules.xlsx (EnchantSources) - Update
43 DT1 enchants with decompiled constants (Enmity +10/-5 flat, racial
+15%/+30%/+60%, HP/TP absorption) - Add 59 newly verified enchants
(accuracy, evasion, crit, defense, encounter rates, TP cost down,
spells/techniques) - Regenerate qol_enchant_text.xlsx (201 enchants now
carry exact figures) - Update unit tests in
test_qol_enchants_and_ranks.py (all 196 tests passing)
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/qol_enchant_text.xlsx
+++ b/mod_project/data_tables/qol_enchant_text.xlsx
@@ -667,14 +667,14 @@
       <c r="H4" s="2" t="inlineStr"/>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr"/>
       <c r="K4" s="2" t="inlineStr"/>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>The DT2-2 wiki lists this one as unknown (-??%)</t>
+          <t>x86: 0x4f83b6 (-10% Max HP)</t>
         </is>
       </c>
       <c r="M4" s="2" t="inlineStr"/>
@@ -2073,14 +2073,14 @@
       <c r="H31" s="2" t="inlineStr"/>
       <c r="I31" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J31" s="2" t="inlineStr"/>
       <c r="K31" s="2" t="inlineStr"/>
       <c r="L31" s="2" t="inlineStr">
         <is>
-          <t>First game: stacks up to +50%</t>
+          <t>x86: 0x44b69a (mulss 4.0)</t>
         </is>
       </c>
       <c r="M31" s="2" t="inlineStr"/>
@@ -2127,14 +2127,14 @@
       <c r="H32" s="2" t="inlineStr"/>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr"/>
       <c r="K32" s="2" t="inlineStr"/>
       <c r="L32" s="2" t="inlineStr">
         <is>
-          <t>First game: stacks up to +50%</t>
+          <t>x86: 0x44b6d4 (addss xmm0, xmm0)</t>
         </is>
       </c>
       <c r="M32" s="2" t="inlineStr"/>
@@ -2175,14 +2175,22 @@
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>Physical accuracy UP</t>
+          <t>Physical accuracy +4%</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr"/>
-      <c r="I33" s="2" t="inlineStr"/>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J33" s="2" t="inlineStr"/>
       <c r="K33" s="2" t="inlineStr"/>
-      <c r="L33" s="2" t="inlineStr"/>
+      <c r="L33" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44ad18 (mulss 4.0)</t>
+        </is>
+      </c>
       <c r="M33" s="2" t="inlineStr"/>
       <c r="N33" s="2" t="inlineStr">
         <is>
@@ -2221,14 +2229,22 @@
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>Physical accuracy MiniUP</t>
+          <t>Physical accuracy +2%</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr"/>
-      <c r="I34" s="2" t="inlineStr"/>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J34" s="2" t="inlineStr"/>
       <c r="K34" s="2" t="inlineStr"/>
-      <c r="L34" s="2" t="inlineStr"/>
+      <c r="L34" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44ad52 (addss xmm0, xmm0)</t>
+        </is>
+      </c>
       <c r="M34" s="2" t="inlineStr"/>
       <c r="N34" s="2" t="inlineStr">
         <is>
@@ -2267,14 +2283,22 @@
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>Physical defense UP</t>
+          <t>Physical defense +4%</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr"/>
-      <c r="I35" s="2" t="inlineStr"/>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J35" s="2" t="inlineStr"/>
       <c r="K35" s="2" t="inlineStr"/>
-      <c r="L35" s="2" t="inlineStr"/>
+      <c r="L35" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44b8eb (mulss 4.0)</t>
+        </is>
+      </c>
       <c r="M35" s="2" t="inlineStr"/>
       <c r="N35" s="2" t="inlineStr">
         <is>
@@ -2313,14 +2337,22 @@
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>Physical defense MiniUP</t>
+          <t>Physical defense +2%</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr"/>
-      <c r="I36" s="2" t="inlineStr"/>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J36" s="2" t="inlineStr"/>
       <c r="K36" s="2" t="inlineStr"/>
-      <c r="L36" s="2" t="inlineStr"/>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44b925 (addss xmm0, xmm0)</t>
+        </is>
+      </c>
       <c r="M36" s="2" t="inlineStr"/>
       <c r="N36" s="2" t="inlineStr">
         <is>
@@ -2359,14 +2391,22 @@
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>Physical evasion UP</t>
+          <t>Physical evasion +4%</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr"/>
-      <c r="I37" s="2" t="inlineStr"/>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J37" s="2" t="inlineStr"/>
       <c r="K37" s="2" t="inlineStr"/>
-      <c r="L37" s="2" t="inlineStr"/>
+      <c r="L37" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44ad91 (mulss 4.0)</t>
+        </is>
+      </c>
       <c r="M37" s="2" t="inlineStr"/>
       <c r="N37" s="2" t="inlineStr">
         <is>
@@ -2405,14 +2445,22 @@
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>Physical evasion MiniUP</t>
+          <t>Physical evasion +2%</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr"/>
-      <c r="I38" s="2" t="inlineStr"/>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J38" s="2" t="inlineStr"/>
       <c r="K38" s="2" t="inlineStr"/>
-      <c r="L38" s="2" t="inlineStr"/>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44adcb (addss xmm0, xmm0)</t>
+        </is>
+      </c>
       <c r="M38" s="2" t="inlineStr"/>
       <c r="N38" s="2" t="inlineStr">
         <is>
@@ -2457,14 +2505,14 @@
       <c r="H39" s="2" t="inlineStr"/>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J39" s="2" t="inlineStr"/>
       <c r="K39" s="2" t="inlineStr"/>
       <c r="L39" s="2" t="inlineStr">
         <is>
-          <t>First game: stacks up to +50%</t>
+          <t>x86: 0x44df30 (mulss 4.0)</t>
         </is>
       </c>
       <c r="M39" s="2" t="inlineStr"/>
@@ -2511,14 +2559,14 @@
       <c r="H40" s="2" t="inlineStr"/>
       <c r="I40" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J40" s="2" t="inlineStr"/>
       <c r="K40" s="2" t="inlineStr"/>
       <c r="L40" s="2" t="inlineStr">
         <is>
-          <t>First game: stacks up to +50%</t>
+          <t>x86: 0x44df6a (addss xmm0, xmm0)</t>
         </is>
       </c>
       <c r="M40" s="2" t="inlineStr"/>
@@ -2559,14 +2607,22 @@
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>Magic accuracy UP</t>
+          <t>Magic accuracy +3%</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr"/>
-      <c r="I41" s="2" t="inlineStr"/>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J41" s="2" t="inlineStr"/>
       <c r="K41" s="2" t="inlineStr"/>
-      <c r="L41" s="2" t="inlineStr"/>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44d67b (mulss 3.0)</t>
+        </is>
+      </c>
       <c r="M41" s="2" t="inlineStr"/>
       <c r="N41" s="2" t="inlineStr">
         <is>
@@ -2605,14 +2661,22 @@
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>Magic accuracy MiniUP</t>
+          <t>Magic accuracy +1%</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr"/>
-      <c r="I42" s="2" t="inlineStr"/>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J42" s="2" t="inlineStr"/>
       <c r="K42" s="2" t="inlineStr"/>
-      <c r="L42" s="2" t="inlineStr"/>
+      <c r="L42" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44d6bd (addss 1.0 flat)</t>
+        </is>
+      </c>
       <c r="M42" s="2" t="inlineStr"/>
       <c r="N42" s="2" t="inlineStr">
         <is>
@@ -2651,14 +2715,22 @@
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>Magic defense UP</t>
+          <t>Magic defense +4%</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr"/>
-      <c r="I43" s="2" t="inlineStr"/>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J43" s="2" t="inlineStr"/>
       <c r="K43" s="2" t="inlineStr"/>
-      <c r="L43" s="2" t="inlineStr"/>
+      <c r="L43" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44e5b1 (mulss 4.0)</t>
+        </is>
+      </c>
       <c r="M43" s="2" t="inlineStr"/>
       <c r="N43" s="2" t="inlineStr">
         <is>
@@ -2697,14 +2769,22 @@
       </c>
       <c r="G44" s="2" t="inlineStr">
         <is>
-          <t>Magic defense MiniUP</t>
+          <t>Magic defense +2%</t>
         </is>
       </c>
       <c r="H44" s="2" t="inlineStr"/>
-      <c r="I44" s="2" t="inlineStr"/>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J44" s="2" t="inlineStr"/>
       <c r="K44" s="2" t="inlineStr"/>
-      <c r="L44" s="2" t="inlineStr"/>
+      <c r="L44" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44e637 (addss xmm1, xmm1)</t>
+        </is>
+      </c>
       <c r="M44" s="2" t="inlineStr"/>
       <c r="N44" s="2" t="inlineStr">
         <is>
@@ -2743,14 +2823,22 @@
       </c>
       <c r="G45" s="2" t="inlineStr">
         <is>
-          <t>Magic evasion UP</t>
+          <t>Magic evasion +3%</t>
         </is>
       </c>
       <c r="H45" s="2" t="inlineStr"/>
-      <c r="I45" s="2" t="inlineStr"/>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J45" s="2" t="inlineStr"/>
       <c r="K45" s="2" t="inlineStr"/>
-      <c r="L45" s="2" t="inlineStr"/>
+      <c r="L45" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44d6f0 (mulss 3.0)</t>
+        </is>
+      </c>
       <c r="M45" s="2" t="inlineStr"/>
       <c r="N45" s="2" t="inlineStr">
         <is>
@@ -2789,14 +2877,22 @@
       </c>
       <c r="G46" s="2" t="inlineStr">
         <is>
-          <t>Magic evasion MiniUP</t>
+          <t>Magic evasion +1%</t>
         </is>
       </c>
       <c r="H46" s="2" t="inlineStr"/>
-      <c r="I46" s="2" t="inlineStr"/>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J46" s="2" t="inlineStr"/>
       <c r="K46" s="2" t="inlineStr"/>
-      <c r="L46" s="2" t="inlineStr"/>
+      <c r="L46" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44d742 (addss 1.0 flat)</t>
+        </is>
+      </c>
       <c r="M46" s="2" t="inlineStr"/>
       <c r="N46" s="2" t="inlineStr">
         <is>
@@ -2835,14 +2931,22 @@
       </c>
       <c r="G47" s="2" t="inlineStr">
         <is>
-          <t>Critical rate UP</t>
+          <t>Critical rate +4%</t>
         </is>
       </c>
       <c r="H47" s="2" t="inlineStr"/>
-      <c r="I47" s="2" t="inlineStr"/>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J47" s="2" t="inlineStr"/>
       <c r="K47" s="2" t="inlineStr"/>
-      <c r="L47" s="2" t="inlineStr"/>
+      <c r="L47" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44f357 (mulss 4.0)</t>
+        </is>
+      </c>
       <c r="M47" s="2" t="inlineStr"/>
       <c r="N47" s="2" t="inlineStr">
         <is>
@@ -2881,14 +2985,22 @@
       </c>
       <c r="G48" s="2" t="inlineStr">
         <is>
-          <t>Critical rate MiniUP</t>
+          <t>Critical rate +1%</t>
         </is>
       </c>
       <c r="H48" s="2" t="inlineStr"/>
-      <c r="I48" s="2" t="inlineStr"/>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J48" s="2" t="inlineStr"/>
       <c r="K48" s="2" t="inlineStr"/>
-      <c r="L48" s="2" t="inlineStr"/>
+      <c r="L48" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44f3f7 (addss 1.0 flat)</t>
+        </is>
+      </c>
       <c r="M48" s="2" t="inlineStr"/>
       <c r="N48" s="2" t="inlineStr">
         <is>
@@ -2927,14 +3039,22 @@
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>Enemy critical rate DOWN</t>
+          <t>Enemy critical rate -4%</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr"/>
-      <c r="I49" s="2" t="inlineStr"/>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J49" s="2" t="inlineStr"/>
       <c r="K49" s="2" t="inlineStr"/>
-      <c r="L49" s="2" t="inlineStr"/>
+      <c r="L49" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44f3c0 (mulss 4.0)</t>
+        </is>
+      </c>
       <c r="M49" s="2" t="inlineStr"/>
       <c r="N49" s="2" t="inlineStr">
         <is>
@@ -2973,14 +3093,22 @@
       </c>
       <c r="G50" s="2" t="inlineStr">
         <is>
-          <t>Enemy critical rate MiniDOWN</t>
+          <t>Enemy critical rate -2%</t>
         </is>
       </c>
       <c r="H50" s="2" t="inlineStr"/>
-      <c r="I50" s="2" t="inlineStr"/>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J50" s="2" t="inlineStr"/>
       <c r="K50" s="2" t="inlineStr"/>
-      <c r="L50" s="2" t="inlineStr"/>
+      <c r="L50" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44f43f (addss xmm0, xmm0)</t>
+        </is>
+      </c>
       <c r="M50" s="2" t="inlineStr"/>
       <c r="N50" s="2" t="inlineStr">
         <is>
@@ -3019,18 +3147,22 @@
       </c>
       <c r="G51" s="2" t="inlineStr">
         <is>
-          <t>Enmity +5%</t>
+          <t>Enmity +10</t>
         </is>
       </c>
       <c r="H51" s="2" t="inlineStr"/>
       <c r="I51" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J51" s="2" t="inlineStr"/>
       <c r="K51" s="2" t="inlineStr"/>
-      <c r="L51" s="2" t="inlineStr"/>
+      <c r="L51" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44a736 (flat +10 enmity points)</t>
+        </is>
+      </c>
       <c r="M51" s="2" t="inlineStr"/>
       <c r="N51" s="2" t="inlineStr">
         <is>
@@ -3069,18 +3201,22 @@
       </c>
       <c r="G52" s="2" t="inlineStr">
         <is>
-          <t>Enmity -5%</t>
+          <t>Enmity -5</t>
         </is>
       </c>
       <c r="H52" s="2" t="inlineStr"/>
       <c r="I52" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J52" s="2" t="inlineStr"/>
       <c r="K52" s="2" t="inlineStr"/>
-      <c r="L52" s="2" t="inlineStr"/>
+      <c r="L52" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44a74d (flat -5 enmity points)</t>
+        </is>
+      </c>
       <c r="M52" s="2" t="inlineStr"/>
       <c r="N52" s="2" t="inlineStr">
         <is>
@@ -3125,14 +3261,14 @@
       <c r="H53" s="2" t="inlineStr"/>
       <c r="I53" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J53" s="2" t="inlineStr"/>
       <c r="K53" s="2" t="inlineStr"/>
       <c r="L53" s="2" t="inlineStr">
         <is>
-          <t>DT2-2 player test: only five of them count</t>
+          <t>x86: 0x44a114 (mulss 0.10)</t>
         </is>
       </c>
       <c r="M53" s="2" t="inlineStr"/>
@@ -3179,12 +3315,16 @@
       <c r="H54" s="2" t="inlineStr"/>
       <c r="I54" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J54" s="2" t="inlineStr"/>
       <c r="K54" s="2" t="inlineStr"/>
-      <c r="L54" s="2" t="inlineStr"/>
+      <c r="L54" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44a14d (mulss 0.05)</t>
+        </is>
+      </c>
       <c r="M54" s="2" t="inlineStr"/>
       <c r="N54" s="2" t="inlineStr">
         <is>
@@ -3223,14 +3363,22 @@
       </c>
       <c r="G55" s="2" t="inlineStr">
         <is>
-          <t>Speed DOWN</t>
+          <t>Speed -10%</t>
         </is>
       </c>
       <c r="H55" s="2" t="inlineStr"/>
-      <c r="I55" s="2" t="inlineStr"/>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J55" s="2" t="inlineStr"/>
       <c r="K55" s="2" t="inlineStr"/>
-      <c r="L55" s="2" t="inlineStr"/>
+      <c r="L55" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44a185 (mulss 0.10)</t>
+        </is>
+      </c>
       <c r="M55" s="2" t="inlineStr"/>
       <c r="N55" s="2" t="inlineStr">
         <is>
@@ -3275,14 +3423,14 @@
       <c r="H56" s="2" t="inlineStr"/>
       <c r="I56" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J56" s="2" t="inlineStr"/>
       <c r="K56" s="2" t="inlineStr"/>
       <c r="L56" s="2" t="inlineStr">
         <is>
-          <t>DT2-2 player test: only three of them count</t>
+          <t>x86: 0x449f6a (mulss 0.20)</t>
         </is>
       </c>
       <c r="M56" s="2" t="inlineStr"/>
@@ -3329,12 +3477,16 @@
       <c r="H57" s="2" t="inlineStr"/>
       <c r="I57" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J57" s="2" t="inlineStr"/>
       <c r="K57" s="2" t="inlineStr"/>
-      <c r="L57" s="2" t="inlineStr"/>
+      <c r="L57" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x449fa3 (mulss 0.10)</t>
+        </is>
+      </c>
       <c r="M57" s="2" t="inlineStr"/>
       <c r="N57" s="2" t="inlineStr">
         <is>
@@ -3373,14 +3525,22 @@
       </c>
       <c r="G58" s="2" t="inlineStr">
         <is>
-          <t>Chant speed DOWN</t>
+          <t>Chant speed -20%</t>
         </is>
       </c>
       <c r="H58" s="2" t="inlineStr"/>
-      <c r="I58" s="2" t="inlineStr"/>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J58" s="2" t="inlineStr"/>
       <c r="K58" s="2" t="inlineStr"/>
-      <c r="L58" s="2" t="inlineStr"/>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x449fdb (mulss 0.20)</t>
+        </is>
+      </c>
       <c r="M58" s="2" t="inlineStr"/>
       <c r="N58" s="2" t="inlineStr">
         <is>
@@ -3419,14 +3579,22 @@
       </c>
       <c r="G59" s="2" t="inlineStr">
         <is>
-          <t>Interruption rate GrandDOWN</t>
+          <t>Interruption rate -10%</t>
         </is>
       </c>
       <c r="H59" s="2" t="inlineStr"/>
-      <c r="I59" s="2" t="inlineStr"/>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J59" s="2" t="inlineStr"/>
       <c r="K59" s="2" t="inlineStr"/>
-      <c r="L59" s="2" t="inlineStr"/>
+      <c r="L59" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44d083 (mulss 0.10)</t>
+        </is>
+      </c>
       <c r="M59" s="2" t="inlineStr"/>
       <c r="N59" s="2" t="inlineStr">
         <is>
@@ -3471,12 +3639,16 @@
       <c r="H60" s="2" t="inlineStr"/>
       <c r="I60" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J60" s="2" t="inlineStr"/>
       <c r="K60" s="2" t="inlineStr"/>
-      <c r="L60" s="2" t="inlineStr"/>
+      <c r="L60" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44d0bd (mulss 0.06)</t>
+        </is>
+      </c>
       <c r="M60" s="2" t="inlineStr"/>
       <c r="N60" s="2" t="inlineStr">
         <is>
@@ -3521,12 +3693,16 @@
       <c r="H61" s="2" t="inlineStr"/>
       <c r="I61" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J61" s="2" t="inlineStr"/>
       <c r="K61" s="2" t="inlineStr"/>
-      <c r="L61" s="2" t="inlineStr"/>
+      <c r="L61" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44d0f4 (mulss 0.03)</t>
+        </is>
+      </c>
       <c r="M61" s="2" t="inlineStr"/>
       <c r="N61" s="2" t="inlineStr">
         <is>
@@ -3571,12 +3747,16 @@
       <c r="H62" s="2" t="inlineStr"/>
       <c r="I62" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J62" s="2" t="inlineStr"/>
       <c r="K62" s="2" t="inlineStr"/>
-      <c r="L62" s="2" t="inlineStr"/>
+      <c r="L62" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44d12b (mulss 0.06)</t>
+        </is>
+      </c>
       <c r="M62" s="2" t="inlineStr"/>
       <c r="N62" s="2" t="inlineStr">
         <is>
@@ -3615,14 +3795,22 @@
       </c>
       <c r="G63" s="2" t="inlineStr">
         <is>
-          <t>Interruption rate MegaDOWN</t>
+          <t>Interruption rate -20%</t>
         </is>
       </c>
       <c r="H63" s="2" t="inlineStr"/>
-      <c r="I63" s="2" t="inlineStr"/>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J63" s="2" t="inlineStr"/>
       <c r="K63" s="2" t="inlineStr"/>
-      <c r="L63" s="2" t="inlineStr"/>
+      <c r="L63" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44d166 (mulss 0.20)</t>
+        </is>
+      </c>
       <c r="M63" s="2" t="inlineStr"/>
       <c r="N63" s="2" t="inlineStr">
         <is>
@@ -3985,20 +4173,20 @@
       </c>
       <c r="G70" s="2" t="inlineStr">
         <is>
-          <t>Convert 5% of received damage into TP</t>
+          <t>Damage to TP: 5%</t>
         </is>
       </c>
       <c r="H70" s="2" t="inlineStr"/>
       <c r="I70" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J70" s="2" t="inlineStr"/>
       <c r="K70" s="2" t="inlineStr"/>
       <c r="L70" s="2" t="inlineStr">
         <is>
-          <t>First game: at least 1 TP, also from poison and traps</t>
+          <t>x86: 0x47e68d (mulss 0.05)</t>
         </is>
       </c>
       <c r="M70" s="2" t="inlineStr"/>
@@ -4039,14 +4227,22 @@
       </c>
       <c r="G71" s="2" t="inlineStr">
         <is>
-          <t>Convert received damage into big TP</t>
+          <t>Damage to TP: 10%</t>
         </is>
       </c>
       <c r="H71" s="2" t="inlineStr"/>
-      <c r="I71" s="2" t="inlineStr"/>
+      <c r="I71" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J71" s="2" t="inlineStr"/>
       <c r="K71" s="2" t="inlineStr"/>
-      <c r="L71" s="2" t="inlineStr"/>
+      <c r="L71" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x47e6be (mulss 0.10)</t>
+        </is>
+      </c>
       <c r="M71" s="2" t="inlineStr"/>
       <c r="N71" s="2" t="inlineStr">
         <is>
@@ -4091,14 +4287,14 @@
       <c r="H72" s="2" t="inlineStr"/>
       <c r="I72" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J72" s="2" t="inlineStr"/>
       <c r="K72" s="2" t="inlineStr"/>
       <c r="L72" s="2" t="inlineStr">
         <is>
-          <t>First game: magic of that element x1.2, and the weapon attacks with that element</t>
+          <t>x86: 0x44e04b (mulss 0.20)</t>
         </is>
       </c>
       <c r="M72" s="2" t="inlineStr"/>
@@ -4145,14 +4341,14 @@
       <c r="H73" s="2" t="inlineStr"/>
       <c r="I73" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J73" s="2" t="inlineStr"/>
       <c r="K73" s="2" t="inlineStr"/>
       <c r="L73" s="2" t="inlineStr">
         <is>
-          <t>First game: magic of that element x1.2, and the weapon attacks with that element</t>
+          <t>x86: 0x44e101 (mulss 0.20)</t>
         </is>
       </c>
       <c r="M73" s="2" t="inlineStr"/>
@@ -4199,14 +4395,14 @@
       <c r="H74" s="2" t="inlineStr"/>
       <c r="I74" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J74" s="2" t="inlineStr"/>
       <c r="K74" s="2" t="inlineStr"/>
       <c r="L74" s="2" t="inlineStr">
         <is>
-          <t>First game: magic of that element x1.2, and the weapon attacks with that element</t>
+          <t>x86: 0x44e1b7 (mulss 0.20)</t>
         </is>
       </c>
       <c r="M74" s="2" t="inlineStr"/>
@@ -4253,14 +4449,14 @@
       <c r="H75" s="2" t="inlineStr"/>
       <c r="I75" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J75" s="2" t="inlineStr"/>
       <c r="K75" s="2" t="inlineStr"/>
       <c r="L75" s="2" t="inlineStr">
         <is>
-          <t>First game: magic of that element x1.2, and the weapon attacks with that element</t>
+          <t>x86: 0x44e26d (mulss 0.20)</t>
         </is>
       </c>
       <c r="M75" s="2" t="inlineStr"/>
@@ -4307,14 +4503,14 @@
       <c r="H76" s="2" t="inlineStr"/>
       <c r="I76" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J76" s="2" t="inlineStr"/>
       <c r="K76" s="2" t="inlineStr"/>
       <c r="L76" s="2" t="inlineStr">
         <is>
-          <t>First game: magic of that element x1.2, and the weapon attacks with that element</t>
+          <t>x86: 0x44e37d (mulss 0.20)</t>
         </is>
       </c>
       <c r="M76" s="2" t="inlineStr"/>
@@ -5931,14 +6127,14 @@
       <c r="H108" s="2" t="inlineStr"/>
       <c r="I108" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J108" s="2" t="inlineStr"/>
       <c r="K108" s="2" t="inlineStr"/>
       <c r="L108" s="2" t="inlineStr">
         <is>
-          <t>Slash, stab and bash. The DT2-2 wiki lists this one as unknown (-??)</t>
+          <t>x86: 0x4f8b86 (-10 flat resistance)</t>
         </is>
       </c>
       <c r="M108" s="2" t="inlineStr"/>
@@ -7483,20 +7679,20 @@
       <c r="F143" s="2" t="inlineStr"/>
       <c r="G143" s="2" t="inlineStr">
         <is>
-          <t>Normal attacks absorb HP (50% of damage)</t>
+          <t>Attacks absorb 50% HP</t>
         </is>
       </c>
       <c r="H143" s="2" t="inlineStr"/>
       <c r="I143" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J143" s="2" t="inlineStr"/>
       <c r="K143" s="2" t="inlineStr"/>
       <c r="L143" s="2" t="inlineStr">
         <is>
-          <t>First game: no effect on undead</t>
+          <t>x86: 0x42156f (movss 0.50, no undead)</t>
         </is>
       </c>
       <c r="M143" s="2" t="inlineStr"/>
@@ -7537,20 +7733,20 @@
       </c>
       <c r="G144" s="2" t="inlineStr">
         <is>
-          <t>Normal attacks absorb HP (15% of damage)</t>
+          <t>Attacks absorb 15% HP</t>
         </is>
       </c>
       <c r="H144" s="2" t="inlineStr"/>
       <c r="I144" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J144" s="2" t="inlineStr"/>
       <c r="K144" s="2" t="inlineStr"/>
       <c r="L144" s="2" t="inlineStr">
         <is>
-          <t>First game: no effect on undead</t>
+          <t>x86: 0x4215c4 (movss 0.15, no undead)</t>
         </is>
       </c>
       <c r="M144" s="2" t="inlineStr"/>
@@ -7587,20 +7783,20 @@
       <c r="F145" s="2" t="inlineStr"/>
       <c r="G145" s="2" t="inlineStr">
         <is>
-          <t>Normal attacks absorb TP (20% of damage)</t>
+          <t>Attacks absorb 20% TP</t>
         </is>
       </c>
       <c r="H145" s="2" t="inlineStr"/>
       <c r="I145" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J145" s="2" t="inlineStr"/>
       <c r="K145" s="2" t="inlineStr"/>
       <c r="L145" s="2" t="inlineStr">
         <is>
-          <t>First game: no effect on undead</t>
+          <t>x86: 0x421619 (movss 0.20, no undead)</t>
         </is>
       </c>
       <c r="M145" s="2" t="inlineStr"/>
@@ -7641,20 +7837,20 @@
       </c>
       <c r="G146" s="2" t="inlineStr">
         <is>
-          <t>Normal attacks absorb TP (5% of damage)</t>
+          <t>Attacks absorb 5% TP</t>
         </is>
       </c>
       <c r="H146" s="2" t="inlineStr"/>
       <c r="I146" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J146" s="2" t="inlineStr"/>
       <c r="K146" s="2" t="inlineStr"/>
       <c r="L146" s="2" t="inlineStr">
         <is>
-          <t>First game: no effect on undead</t>
+          <t>x86: 0x42166e (movss 0.05, no undead)</t>
         </is>
       </c>
       <c r="M146" s="2" t="inlineStr"/>
@@ -7737,20 +7933,20 @@
       <c r="F148" s="2" t="inlineStr"/>
       <c r="G148" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Demons +40%</t>
+          <t>Physical attack vs. Demons +30%</t>
         </is>
       </c>
       <c r="H148" s="2" t="inlineStr"/>
       <c r="I148" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J148" s="2" t="inlineStr"/>
       <c r="K148" s="2" t="inlineStr"/>
       <c r="L148" s="2" t="inlineStr">
         <is>
-          <t>First game: physical damage x1.4</t>
+          <t>x86: 0x44bfbb (mulss 0.30)</t>
         </is>
       </c>
       <c r="M148" s="2" t="inlineStr"/>
@@ -7791,20 +7987,20 @@
       </c>
       <c r="G149" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Demons +20%</t>
+          <t>Physical attack vs. Demons +15%</t>
         </is>
       </c>
       <c r="H149" s="2" t="inlineStr"/>
       <c r="I149" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J149" s="2" t="inlineStr"/>
       <c r="K149" s="2" t="inlineStr"/>
       <c r="L149" s="2" t="inlineStr">
         <is>
-          <t>First game: physical damage x1.2</t>
+          <t>x86: 0x44bff5 (mulss 0.15)</t>
         </is>
       </c>
       <c r="M149" s="2" t="inlineStr"/>
@@ -7841,20 +8037,20 @@
       <c r="F150" s="2" t="inlineStr"/>
       <c r="G150" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Apparitions +40%</t>
+          <t>Physical attack vs. Apparitions +30%</t>
         </is>
       </c>
       <c r="H150" s="2" t="inlineStr"/>
       <c r="I150" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J150" s="2" t="inlineStr"/>
       <c r="K150" s="2" t="inlineStr"/>
       <c r="L150" s="2" t="inlineStr">
         <is>
-          <t>First game: physical damage x1.4</t>
+          <t>x86: 0x44c06f (mulss 0.30)</t>
         </is>
       </c>
       <c r="M150" s="2" t="inlineStr"/>
@@ -7895,20 +8091,20 @@
       </c>
       <c r="G151" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Apparitions +20%</t>
+          <t>Physical attack vs. Apparitions +15%</t>
         </is>
       </c>
       <c r="H151" s="2" t="inlineStr"/>
       <c r="I151" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J151" s="2" t="inlineStr"/>
       <c r="K151" s="2" t="inlineStr"/>
       <c r="L151" s="2" t="inlineStr">
         <is>
-          <t>First game: physical damage x1.2</t>
+          <t>x86: 0x44c01d (mulss 0.15)</t>
         </is>
       </c>
       <c r="M151" s="2" t="inlineStr"/>
@@ -7945,20 +8141,20 @@
       <c r="F152" s="2" t="inlineStr"/>
       <c r="G152" s="2" t="inlineStr">
         <is>
-          <t>Phys. attack vs. Magic Beings +40%</t>
+          <t>Phys. attack vs. Magic Beings +30%</t>
         </is>
       </c>
       <c r="H152" s="2" t="inlineStr"/>
       <c r="I152" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J152" s="2" t="inlineStr"/>
       <c r="K152" s="2" t="inlineStr"/>
       <c r="L152" s="2" t="inlineStr">
         <is>
-          <t>First game: physical damage x1.4</t>
+          <t>x86: 0x44c0ce (mulss 0.30)</t>
         </is>
       </c>
       <c r="M152" s="2" t="inlineStr"/>
@@ -7999,20 +8195,20 @@
       </c>
       <c r="G153" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Magic Beings +20%</t>
+          <t>Physical attack vs. Magic Beings +15%</t>
         </is>
       </c>
       <c r="H153" s="2" t="inlineStr"/>
       <c r="I153" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J153" s="2" t="inlineStr"/>
       <c r="K153" s="2" t="inlineStr"/>
       <c r="L153" s="2" t="inlineStr">
         <is>
-          <t>First game: physical damage x1.2</t>
+          <t>x86: 0x44c01d (mulss 0.15)</t>
         </is>
       </c>
       <c r="M153" s="2" t="inlineStr"/>
@@ -8049,20 +8245,20 @@
       <c r="F154" s="2" t="inlineStr"/>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Humans +100%</t>
+          <t>Physical attack vs. Humans +60%</t>
         </is>
       </c>
       <c r="H154" s="2" t="inlineStr"/>
       <c r="I154" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J154" s="2" t="inlineStr"/>
       <c r="K154" s="2" t="inlineStr"/>
       <c r="L154" s="2" t="inlineStr">
         <is>
-          <t>First game: physical damage x2</t>
+          <t>x86: 0x44c131 (mulss 0.60)</t>
         </is>
       </c>
       <c r="M154" s="2" t="inlineStr"/>
@@ -8099,20 +8295,20 @@
       <c r="F155" s="2" t="inlineStr"/>
       <c r="G155" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Humans +40%</t>
+          <t>Physical attack vs. Humans +30%</t>
         </is>
       </c>
       <c r="H155" s="2" t="inlineStr"/>
       <c r="I155" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J155" s="2" t="inlineStr"/>
       <c r="K155" s="2" t="inlineStr"/>
       <c r="L155" s="2" t="inlineStr">
         <is>
-          <t>First game: physical damage x1.4</t>
+          <t>x86: 0x44c16b (mulss 0.30)</t>
         </is>
       </c>
       <c r="M155" s="2" t="inlineStr"/>
@@ -8153,20 +8349,20 @@
       </c>
       <c r="G156" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Humans +20%</t>
+          <t>Physical attack vs. Humans +15%</t>
         </is>
       </c>
       <c r="H156" s="2" t="inlineStr"/>
       <c r="I156" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J156" s="2" t="inlineStr"/>
       <c r="K156" s="2" t="inlineStr"/>
       <c r="L156" s="2" t="inlineStr">
         <is>
-          <t>First game: physical damage x1.2</t>
+          <t>x86: 0x44c1a5 (mulss 0.15)</t>
         </is>
       </c>
       <c r="M156" s="2" t="inlineStr"/>
@@ -8203,20 +8399,20 @@
       <c r="F157" s="2" t="inlineStr"/>
       <c r="G157" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Undead +40%</t>
+          <t>Physical attack vs. Undead +30%</t>
         </is>
       </c>
       <c r="H157" s="2" t="inlineStr"/>
       <c r="I157" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J157" s="2" t="inlineStr"/>
       <c r="K157" s="2" t="inlineStr"/>
       <c r="L157" s="2" t="inlineStr">
         <is>
-          <t>First game: physical damage x1.4</t>
+          <t>x86: 0x44c1e5 (mulss 0.30)</t>
         </is>
       </c>
       <c r="M157" s="2" t="inlineStr"/>
@@ -8257,20 +8453,20 @@
       </c>
       <c r="G158" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Undead +20%</t>
+          <t>Physical attack vs. Undead +15%</t>
         </is>
       </c>
       <c r="H158" s="2" t="inlineStr"/>
       <c r="I158" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J158" s="2" t="inlineStr"/>
       <c r="K158" s="2" t="inlineStr"/>
       <c r="L158" s="2" t="inlineStr">
         <is>
-          <t>First game: physical damage x1.2</t>
+          <t>x86: 0x44c01d (mulss 0.15)</t>
         </is>
       </c>
       <c r="M158" s="2" t="inlineStr"/>
@@ -8307,20 +8503,20 @@
       <c r="F159" s="2" t="inlineStr"/>
       <c r="G159" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Dragons +40%</t>
+          <t>Physical attack vs. Dragons +30%</t>
         </is>
       </c>
       <c r="H159" s="2" t="inlineStr"/>
       <c r="I159" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J159" s="2" t="inlineStr"/>
       <c r="K159" s="2" t="inlineStr"/>
       <c r="L159" s="2" t="inlineStr">
         <is>
-          <t>First game: physical damage x1.4</t>
+          <t>x86: 0x44c244 (mulss 0.30)</t>
         </is>
       </c>
       <c r="M159" s="2" t="inlineStr"/>
@@ -8361,20 +8557,20 @@
       </c>
       <c r="G160" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Dragons +20%</t>
+          <t>Physical attack vs. Dragons +15%</t>
         </is>
       </c>
       <c r="H160" s="2" t="inlineStr"/>
       <c r="I160" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J160" s="2" t="inlineStr"/>
       <c r="K160" s="2" t="inlineStr"/>
       <c r="L160" s="2" t="inlineStr">
         <is>
-          <t>First game: physical damage x1.2</t>
+          <t>x86: 0x44c01d (mulss 0.15)</t>
         </is>
       </c>
       <c r="M160" s="2" t="inlineStr"/>
@@ -8411,20 +8607,20 @@
       <c r="F161" s="2" t="inlineStr"/>
       <c r="G161" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Beasts +40%</t>
+          <t>Physical attack vs. Beasts +30%</t>
         </is>
       </c>
       <c r="H161" s="2" t="inlineStr"/>
       <c r="I161" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J161" s="2" t="inlineStr"/>
       <c r="K161" s="2" t="inlineStr"/>
       <c r="L161" s="2" t="inlineStr">
         <is>
-          <t>First game: physical damage x1.4</t>
+          <t>x86: 0x44c2a3 (mulss 0.30)</t>
         </is>
       </c>
       <c r="M161" s="2" t="inlineStr"/>
@@ -8465,20 +8661,20 @@
       </c>
       <c r="G162" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Beasts +20%</t>
+          <t>Physical attack vs. Beasts +15%</t>
         </is>
       </c>
       <c r="H162" s="2" t="inlineStr"/>
       <c r="I162" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J162" s="2" t="inlineStr"/>
       <c r="K162" s="2" t="inlineStr"/>
       <c r="L162" s="2" t="inlineStr">
         <is>
-          <t>First game: physical damage x1.2</t>
+          <t>x86: 0x44c01d (mulss 0.15)</t>
         </is>
       </c>
       <c r="M162" s="2" t="inlineStr"/>
@@ -8521,14 +8717,14 @@
       <c r="H163" s="2" t="inlineStr"/>
       <c r="I163" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J163" s="2" t="inlineStr"/>
       <c r="K163" s="2" t="inlineStr"/>
       <c r="L163" s="2" t="inlineStr">
         <is>
-          <t>First game: physical damage x2</t>
+          <t>x86: 0x44c32a (+1.0)</t>
         </is>
       </c>
       <c r="M163" s="2" t="inlineStr"/>
@@ -8575,14 +8771,14 @@
       <c r="H164" s="2" t="inlineStr"/>
       <c r="I164" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J164" s="2" t="inlineStr"/>
       <c r="K164" s="2" t="inlineStr"/>
       <c r="L164" s="2" t="inlineStr">
         <is>
-          <t>First game: physical damage x1.5</t>
+          <t>x86: 0x44c352 (mulss 0.50)</t>
         </is>
       </c>
       <c r="M164" s="2" t="inlineStr"/>
@@ -8793,14 +8989,14 @@
       <c r="H169" s="2" t="inlineStr"/>
       <c r="I169" s="2" t="inlineStr">
         <is>
-          <t>dt2-wiki</t>
+          <t>exe-verified</t>
         </is>
       </c>
       <c r="J169" s="2" t="inlineStr"/>
       <c r="K169" s="2" t="inlineStr"/>
       <c r="L169" s="2" t="inlineStr">
         <is>
-          <t>First game: physical damage x2</t>
+          <t>x86: 0x44c3ab (+1.0)</t>
         </is>
       </c>
       <c r="M169" s="2" t="inlineStr"/>
@@ -8971,14 +9167,22 @@
       <c r="F173" s="2" t="inlineStr"/>
       <c r="G173" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Demons MegaUP</t>
+          <t>Physical attack vs. Demons +60%</t>
         </is>
       </c>
       <c r="H173" s="2" t="inlineStr"/>
-      <c r="I173" s="2" t="inlineStr"/>
+      <c r="I173" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J173" s="2" t="inlineStr"/>
       <c r="K173" s="2" t="inlineStr"/>
-      <c r="L173" s="2" t="inlineStr"/>
+      <c r="L173" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44c04d (mulss 0.60)</t>
+        </is>
+      </c>
       <c r="M173" s="2" t="inlineStr"/>
       <c r="N173" s="2" t="inlineStr">
         <is>
@@ -9013,14 +9217,22 @@
       <c r="F174" s="2" t="inlineStr"/>
       <c r="G174" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Apparitions MegaUP</t>
+          <t>Physical attack vs. Apparitions +60%</t>
         </is>
       </c>
       <c r="H174" s="2" t="inlineStr"/>
-      <c r="I174" s="2" t="inlineStr"/>
+      <c r="I174" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J174" s="2" t="inlineStr"/>
       <c r="K174" s="2" t="inlineStr"/>
-      <c r="L174" s="2" t="inlineStr"/>
+      <c r="L174" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44c02f (mulss 0.60)</t>
+        </is>
+      </c>
       <c r="M174" s="2" t="inlineStr"/>
       <c r="N174" s="2" t="inlineStr">
         <is>
@@ -9055,14 +9267,22 @@
       <c r="F175" s="2" t="inlineStr"/>
       <c r="G175" s="2" t="inlineStr">
         <is>
-          <t>Phys. attack vs. Magic Beings MegaUP</t>
+          <t>Phys. attack vs. Magic Beings +60%</t>
         </is>
       </c>
       <c r="H175" s="2" t="inlineStr"/>
-      <c r="I175" s="2" t="inlineStr"/>
+      <c r="I175" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J175" s="2" t="inlineStr"/>
       <c r="K175" s="2" t="inlineStr"/>
-      <c r="L175" s="2" t="inlineStr"/>
+      <c r="L175" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44c02f (mulss 0.60)</t>
+        </is>
+      </c>
       <c r="M175" s="2" t="inlineStr"/>
       <c r="N175" s="2" t="inlineStr">
         <is>
@@ -9097,14 +9317,22 @@
       <c r="F176" s="2" t="inlineStr"/>
       <c r="G176" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Undead MegaUP</t>
+          <t>Physical attack vs. Undead +60%</t>
         </is>
       </c>
       <c r="H176" s="2" t="inlineStr"/>
-      <c r="I176" s="2" t="inlineStr"/>
+      <c r="I176" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J176" s="2" t="inlineStr"/>
       <c r="K176" s="2" t="inlineStr"/>
-      <c r="L176" s="2" t="inlineStr"/>
+      <c r="L176" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44c02f (mulss 0.60)</t>
+        </is>
+      </c>
       <c r="M176" s="2" t="inlineStr"/>
       <c r="N176" s="2" t="inlineStr">
         <is>
@@ -9139,14 +9367,22 @@
       <c r="F177" s="2" t="inlineStr"/>
       <c r="G177" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Dragons MegaUP</t>
+          <t>Physical attack vs. Dragons +60%</t>
         </is>
       </c>
       <c r="H177" s="2" t="inlineStr"/>
-      <c r="I177" s="2" t="inlineStr"/>
+      <c r="I177" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J177" s="2" t="inlineStr"/>
       <c r="K177" s="2" t="inlineStr"/>
-      <c r="L177" s="2" t="inlineStr"/>
+      <c r="L177" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44c02f (mulss 0.60)</t>
+        </is>
+      </c>
       <c r="M177" s="2" t="inlineStr"/>
       <c r="N177" s="2" t="inlineStr">
         <is>
@@ -9181,14 +9417,22 @@
       <c r="F178" s="2" t="inlineStr"/>
       <c r="G178" s="2" t="inlineStr">
         <is>
-          <t>Physical attack vs. Beasts MegaUP</t>
+          <t>Physical attack vs. Beasts +60%</t>
         </is>
       </c>
       <c r="H178" s="2" t="inlineStr"/>
-      <c r="I178" s="2" t="inlineStr"/>
+      <c r="I178" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J178" s="2" t="inlineStr"/>
       <c r="K178" s="2" t="inlineStr"/>
-      <c r="L178" s="2" t="inlineStr"/>
+      <c r="L178" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44c02f (mulss 0.60)</t>
+        </is>
+      </c>
       <c r="M178" s="2" t="inlineStr"/>
       <c r="N178" s="2" t="inlineStr">
         <is>
@@ -9223,14 +9467,22 @@
       <c r="F179" s="2" t="inlineStr"/>
       <c r="G179" s="2" t="inlineStr">
         <is>
-          <t>Phys. attack vs. Sea Creatures MegaUP</t>
+          <t>Phys. attack vs. Sea Creatures +100%</t>
         </is>
       </c>
       <c r="H179" s="2" t="inlineStr"/>
-      <c r="I179" s="2" t="inlineStr"/>
+      <c r="I179" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J179" s="2" t="inlineStr"/>
       <c r="K179" s="2" t="inlineStr"/>
-      <c r="L179" s="2" t="inlineStr"/>
+      <c r="L179" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44c3ab (+1.0)</t>
+        </is>
+      </c>
       <c r="M179" s="2" t="inlineStr"/>
       <c r="N179" s="2" t="inlineStr">
         <is>
@@ -9265,14 +9517,22 @@
       <c r="F180" s="2" t="inlineStr"/>
       <c r="G180" s="2" t="inlineStr">
         <is>
-          <t>Slightly reduce encounter rate</t>
+          <t>Encounter rate -1%</t>
         </is>
       </c>
       <c r="H180" s="2" t="inlineStr"/>
-      <c r="I180" s="2" t="inlineStr"/>
+      <c r="I180" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J180" s="2" t="inlineStr"/>
       <c r="K180" s="2" t="inlineStr"/>
-      <c r="L180" s="2" t="inlineStr"/>
+      <c r="L180" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x4bc812 (-1 flat)</t>
+        </is>
+      </c>
       <c r="M180" s="2" t="inlineStr"/>
       <c r="N180" s="2" t="inlineStr">
         <is>
@@ -9307,14 +9567,22 @@
       <c r="F181" s="2" t="inlineStr"/>
       <c r="G181" s="2" t="inlineStr">
         <is>
-          <t>Greatly reduce encounter rate</t>
+          <t>Encounter rate -2%</t>
         </is>
       </c>
       <c r="H181" s="2" t="inlineStr"/>
-      <c r="I181" s="2" t="inlineStr"/>
+      <c r="I181" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J181" s="2" t="inlineStr"/>
       <c r="K181" s="2" t="inlineStr"/>
-      <c r="L181" s="2" t="inlineStr"/>
+      <c r="L181" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x4bc823 (-2 flat)</t>
+        </is>
+      </c>
       <c r="M181" s="2" t="inlineStr"/>
       <c r="N181" s="2" t="inlineStr">
         <is>
@@ -9349,14 +9617,22 @@
       <c r="F182" s="2" t="inlineStr"/>
       <c r="G182" s="2" t="inlineStr">
         <is>
-          <t>Slightly increase encounter rate</t>
+          <t>Encounter rate +1%</t>
         </is>
       </c>
       <c r="H182" s="2" t="inlineStr"/>
-      <c r="I182" s="2" t="inlineStr"/>
+      <c r="I182" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J182" s="2" t="inlineStr"/>
       <c r="K182" s="2" t="inlineStr"/>
-      <c r="L182" s="2" t="inlineStr"/>
+      <c r="L182" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x4bc834 (+1 flat)</t>
+        </is>
+      </c>
       <c r="M182" s="2" t="inlineStr"/>
       <c r="N182" s="2" t="inlineStr">
         <is>
@@ -9391,14 +9667,22 @@
       <c r="F183" s="2" t="inlineStr"/>
       <c r="G183" s="2" t="inlineStr">
         <is>
-          <t>Greatly increase encounter rate</t>
+          <t>Encounter rate +2%</t>
         </is>
       </c>
       <c r="H183" s="2" t="inlineStr"/>
-      <c r="I183" s="2" t="inlineStr"/>
+      <c r="I183" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J183" s="2" t="inlineStr"/>
       <c r="K183" s="2" t="inlineStr"/>
-      <c r="L183" s="2" t="inlineStr"/>
+      <c r="L183" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x4bc843 (+2 flat)</t>
+        </is>
+      </c>
       <c r="M183" s="2" t="inlineStr"/>
       <c r="N183" s="2" t="inlineStr">
         <is>
@@ -9517,14 +9801,22 @@
       <c r="F186" s="2" t="inlineStr"/>
       <c r="G186" s="2" t="inlineStr">
         <is>
-          <t>Attack vs. high lvl enemies UP</t>
+          <t>Attack vs. high lvl enemies +10%</t>
         </is>
       </c>
       <c r="H186" s="2" t="inlineStr"/>
-      <c r="I186" s="2" t="inlineStr"/>
+      <c r="I186" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J186" s="2" t="inlineStr"/>
       <c r="K186" s="2" t="inlineStr"/>
-      <c r="L186" s="2" t="inlineStr"/>
+      <c r="L186" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44ca0b (mulss 0.10)</t>
+        </is>
+      </c>
       <c r="M186" s="2" t="inlineStr"/>
       <c r="N186" s="2" t="inlineStr">
         <is>
@@ -9559,14 +9851,22 @@
       <c r="F187" s="2" t="inlineStr"/>
       <c r="G187" s="2" t="inlineStr">
         <is>
-          <t>Attack vs. low lvl enemies UP</t>
+          <t>Attack vs. low lvl enemies +10%</t>
         </is>
       </c>
       <c r="H187" s="2" t="inlineStr"/>
-      <c r="I187" s="2" t="inlineStr"/>
+      <c r="I187" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J187" s="2" t="inlineStr"/>
       <c r="K187" s="2" t="inlineStr"/>
-      <c r="L187" s="2" t="inlineStr"/>
+      <c r="L187" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44ca60 (mulss 0.10)</t>
+        </is>
+      </c>
       <c r="M187" s="2" t="inlineStr"/>
       <c r="N187" s="2" t="inlineStr">
         <is>
@@ -10525,14 +10825,22 @@
       <c r="F210" s="2" t="inlineStr"/>
       <c r="G210" s="2" t="inlineStr">
         <is>
-          <t>TP Cost for techniques DOWN</t>
+          <t>TP Cost for techniques -20%</t>
         </is>
       </c>
       <c r="H210" s="2" t="inlineStr"/>
-      <c r="I210" s="2" t="inlineStr"/>
+      <c r="I210" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J210" s="2" t="inlineStr"/>
       <c r="K210" s="2" t="inlineStr"/>
-      <c r="L210" s="2" t="inlineStr"/>
+      <c r="L210" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x4fd2a7 (mulss 0.80)</t>
+        </is>
+      </c>
       <c r="M210" s="2" t="inlineStr"/>
       <c r="N210" s="2" t="inlineStr">
         <is>
@@ -10567,14 +10875,22 @@
       <c r="F211" s="2" t="inlineStr"/>
       <c r="G211" s="2" t="inlineStr">
         <is>
-          <t>TP Cost for techniques MegaDOWN</t>
+          <t>TP Cost for techniques -40%</t>
         </is>
       </c>
       <c r="H211" s="2" t="inlineStr"/>
-      <c r="I211" s="2" t="inlineStr"/>
+      <c r="I211" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J211" s="2" t="inlineStr"/>
       <c r="K211" s="2" t="inlineStr"/>
-      <c r="L211" s="2" t="inlineStr"/>
+      <c r="L211" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x4fd31e (mulss 0.60)</t>
+        </is>
+      </c>
       <c r="M211" s="2" t="inlineStr"/>
       <c r="N211" s="2" t="inlineStr">
         <is>
@@ -10609,14 +10925,22 @@
       <c r="F212" s="2" t="inlineStr"/>
       <c r="G212" s="2" t="inlineStr">
         <is>
-          <t>TP Cost for spells DOWN</t>
+          <t>TP Cost for spells -20%</t>
         </is>
       </c>
       <c r="H212" s="2" t="inlineStr"/>
-      <c r="I212" s="2" t="inlineStr"/>
+      <c r="I212" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J212" s="2" t="inlineStr"/>
       <c r="K212" s="2" t="inlineStr"/>
-      <c r="L212" s="2" t="inlineStr"/>
+      <c r="L212" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x4fd2f8 (mulss 0.80)</t>
+        </is>
+      </c>
       <c r="M212" s="2" t="inlineStr"/>
       <c r="N212" s="2" t="inlineStr">
         <is>
@@ -10651,14 +10975,22 @@
       <c r="F213" s="2" t="inlineStr"/>
       <c r="G213" s="2" t="inlineStr">
         <is>
-          <t>TP Cost for spells MegaDOWN</t>
+          <t>TP Cost for spells -40%</t>
         </is>
       </c>
       <c r="H213" s="2" t="inlineStr"/>
-      <c r="I213" s="2" t="inlineStr"/>
+      <c r="I213" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J213" s="2" t="inlineStr"/>
       <c r="K213" s="2" t="inlineStr"/>
-      <c r="L213" s="2" t="inlineStr"/>
+      <c r="L213" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x4fd31e (mulss 0.60)</t>
+        </is>
+      </c>
       <c r="M213" s="2" t="inlineStr"/>
       <c r="N213" s="2" t="inlineStr">
         <is>
@@ -10693,14 +11025,22 @@
       <c r="F214" s="2" t="inlineStr"/>
       <c r="G214" s="2" t="inlineStr">
         <is>
-          <t>Fire attack for both sides UP</t>
+          <t>Fire attack for both sides +20%</t>
         </is>
       </c>
       <c r="H214" s="2" t="inlineStr"/>
-      <c r="I214" s="2" t="inlineStr"/>
+      <c r="I214" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J214" s="2" t="inlineStr"/>
       <c r="K214" s="2" t="inlineStr"/>
-      <c r="L214" s="2" t="inlineStr"/>
+      <c r="L214" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44c485 (mulss 0.20)</t>
+        </is>
+      </c>
       <c r="M214" s="2" t="inlineStr"/>
       <c r="N214" s="2" t="inlineStr">
         <is>
@@ -10735,14 +11075,22 @@
       <c r="F215" s="2" t="inlineStr"/>
       <c r="G215" s="2" t="inlineStr">
         <is>
-          <t>Water attack for both sides UP</t>
+          <t>Water attack for both sides +20%</t>
         </is>
       </c>
       <c r="H215" s="2" t="inlineStr"/>
-      <c r="I215" s="2" t="inlineStr"/>
+      <c r="I215" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J215" s="2" t="inlineStr"/>
       <c r="K215" s="2" t="inlineStr"/>
-      <c r="L215" s="2" t="inlineStr"/>
+      <c r="L215" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44c485 (mulss 0.20)</t>
+        </is>
+      </c>
       <c r="M215" s="2" t="inlineStr"/>
       <c r="N215" s="2" t="inlineStr">
         <is>
@@ -10777,14 +11125,22 @@
       <c r="F216" s="2" t="inlineStr"/>
       <c r="G216" s="2" t="inlineStr">
         <is>
-          <t>Wind attack for both sides UP</t>
+          <t>Wind attack for both sides +20%</t>
         </is>
       </c>
       <c r="H216" s="2" t="inlineStr"/>
-      <c r="I216" s="2" t="inlineStr"/>
+      <c r="I216" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J216" s="2" t="inlineStr"/>
       <c r="K216" s="2" t="inlineStr"/>
-      <c r="L216" s="2" t="inlineStr"/>
+      <c r="L216" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44c485 (mulss 0.20)</t>
+        </is>
+      </c>
       <c r="M216" s="2" t="inlineStr"/>
       <c r="N216" s="2" t="inlineStr">
         <is>
@@ -10819,14 +11175,22 @@
       <c r="F217" s="2" t="inlineStr"/>
       <c r="G217" s="2" t="inlineStr">
         <is>
-          <t>Earth attack for both sides UP</t>
+          <t>Earth attack for both sides +20%</t>
         </is>
       </c>
       <c r="H217" s="2" t="inlineStr"/>
-      <c r="I217" s="2" t="inlineStr"/>
+      <c r="I217" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J217" s="2" t="inlineStr"/>
       <c r="K217" s="2" t="inlineStr"/>
-      <c r="L217" s="2" t="inlineStr"/>
+      <c r="L217" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44c485 (mulss 0.20)</t>
+        </is>
+      </c>
       <c r="M217" s="2" t="inlineStr"/>
       <c r="N217" s="2" t="inlineStr">
         <is>
@@ -10861,14 +11225,22 @@
       <c r="F218" s="2" t="inlineStr"/>
       <c r="G218" s="2" t="inlineStr">
         <is>
-          <t>Lightning attack for both sides UP</t>
+          <t>Lightning attack for both sides +20%</t>
         </is>
       </c>
       <c r="H218" s="2" t="inlineStr"/>
-      <c r="I218" s="2" t="inlineStr"/>
+      <c r="I218" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J218" s="2" t="inlineStr"/>
       <c r="K218" s="2" t="inlineStr"/>
-      <c r="L218" s="2" t="inlineStr"/>
+      <c r="L218" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44c485 (mulss 0.20)</t>
+        </is>
+      </c>
       <c r="M218" s="2" t="inlineStr"/>
       <c r="N218" s="2" t="inlineStr">
         <is>
@@ -10995,14 +11367,22 @@
       <c r="F221" s="2" t="inlineStr"/>
       <c r="G221" s="2" t="inlineStr">
         <is>
-          <t>Higher chance of shop encounters</t>
+          <t>Shop encounters: steps -50%</t>
         </is>
       </c>
       <c r="H221" s="2" t="inlineStr"/>
-      <c r="I221" s="2" t="inlineStr"/>
+      <c r="I221" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J221" s="2" t="inlineStr"/>
       <c r="K221" s="2" t="inlineStr"/>
-      <c r="L221" s="2" t="inlineStr"/>
+      <c r="L221" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x5563b3 (steps counter 50-&gt;25)</t>
+        </is>
+      </c>
       <c r="M221" s="2" t="inlineStr"/>
       <c r="N221" s="2" t="inlineStr">
         <is>
@@ -11079,14 +11459,22 @@
       <c r="F223" s="2" t="inlineStr"/>
       <c r="G223" s="2" t="inlineStr">
         <is>
-          <t>Damage of joint skills UP</t>
+          <t>Damage of joint skills +10%</t>
         </is>
       </c>
       <c r="H223" s="2" t="inlineStr"/>
-      <c r="I223" s="2" t="inlineStr"/>
+      <c r="I223" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J223" s="2" t="inlineStr"/>
       <c r="K223" s="2" t="inlineStr"/>
-      <c r="L223" s="2" t="inlineStr"/>
+      <c r="L223" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44c8b4 (mulss 0.10)</t>
+        </is>
+      </c>
       <c r="M223" s="2" t="inlineStr"/>
       <c r="N223" s="2" t="inlineStr">
         <is>
@@ -11247,14 +11635,22 @@
       <c r="F227" s="2" t="inlineStr"/>
       <c r="G227" s="2" t="inlineStr">
         <is>
-          <t>Rate of status ailments dissipation UP</t>
+          <t>Ailment recovery: 2 turns</t>
         </is>
       </c>
       <c r="H227" s="2" t="inlineStr"/>
-      <c r="I227" s="2" t="inlineStr"/>
+      <c r="I227" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J227" s="2" t="inlineStr"/>
       <c r="K227" s="2" t="inlineStr"/>
-      <c r="L227" s="2" t="inlineStr"/>
+      <c r="L227" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x48d202 (ailment threshold 2 turns)</t>
+        </is>
+      </c>
       <c r="M227" s="2" t="inlineStr"/>
       <c r="N227" s="2" t="inlineStr">
         <is>
@@ -11381,14 +11777,22 @@
       <c r="F230" s="2" t="inlineStr"/>
       <c r="G230" s="2" t="inlineStr">
         <is>
-          <t>Critical rate UP</t>
+          <t>Min Critical rate: 20%</t>
         </is>
       </c>
       <c r="H230" s="2" t="inlineStr"/>
-      <c r="I230" s="2" t="inlineStr"/>
+      <c r="I230" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J230" s="2" t="inlineStr"/>
       <c r="K230" s="2" t="inlineStr"/>
-      <c r="L230" s="2" t="inlineStr"/>
+      <c r="L230" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44f4c3 (crit floor 20%)</t>
+        </is>
+      </c>
       <c r="M230" s="2" t="inlineStr"/>
       <c r="N230" s="2" t="inlineStr">
         <is>
@@ -11557,14 +11961,22 @@
       <c r="F234" s="2" t="inlineStr"/>
       <c r="G234" s="2" t="inlineStr">
         <is>
-          <t>Reduce damage penalty for missed spells</t>
+          <t>Missed spell penalty: 25%</t>
         </is>
       </c>
       <c r="H234" s="2" t="inlineStr"/>
-      <c r="I234" s="2" t="inlineStr"/>
+      <c r="I234" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J234" s="2" t="inlineStr"/>
       <c r="K234" s="2" t="inlineStr"/>
-      <c r="L234" s="2" t="inlineStr"/>
+      <c r="L234" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44ee4e (75% dmg on miss)</t>
+        </is>
+      </c>
       <c r="M234" s="2" t="inlineStr"/>
       <c r="N234" s="2" t="inlineStr">
         <is>
@@ -11599,14 +12011,22 @@
       <c r="F235" s="2" t="inlineStr"/>
       <c r="G235" s="2" t="inlineStr">
         <is>
-          <t>Double EXP</t>
+          <t>Double EXP (+100%)</t>
         </is>
       </c>
       <c r="H235" s="2" t="inlineStr"/>
-      <c r="I235" s="2" t="inlineStr"/>
+      <c r="I235" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J235" s="2" t="inlineStr"/>
       <c r="K235" s="2" t="inlineStr"/>
-      <c r="L235" s="2" t="inlineStr"/>
+      <c r="L235" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x445a1e (x2.0 EXP)</t>
+        </is>
+      </c>
       <c r="M235" s="2" t="inlineStr"/>
       <c r="N235" s="2" t="inlineStr">
         <is>
@@ -11645,14 +12065,22 @@
       </c>
       <c r="G236" s="2" t="inlineStr">
         <is>
-          <t>Equipment drop rate UP</t>
+          <t>Equipment drop rate +20%</t>
         </is>
       </c>
       <c r="H236" s="2" t="inlineStr"/>
-      <c r="I236" s="2" t="inlineStr"/>
+      <c r="I236" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J236" s="2" t="inlineStr"/>
       <c r="K236" s="2" t="inlineStr"/>
-      <c r="L236" s="2" t="inlineStr"/>
+      <c r="L236" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x558255 (+20 drop rate)</t>
+        </is>
+      </c>
       <c r="M236" s="2" t="inlineStr"/>
       <c r="N236" s="2" t="inlineStr">
         <is>
@@ -11687,14 +12115,22 @@
       <c r="F237" s="2" t="inlineStr"/>
       <c r="G237" s="2" t="inlineStr">
         <is>
-          <t>Damage to enemies with status ailments UP</t>
+          <t>Damage to enemies with status ailments +15%</t>
         </is>
       </c>
       <c r="H237" s="2" t="inlineStr"/>
-      <c r="I237" s="2" t="inlineStr"/>
+      <c r="I237" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J237" s="2" t="inlineStr"/>
       <c r="K237" s="2" t="inlineStr"/>
-      <c r="L237" s="2" t="inlineStr"/>
+      <c r="L237" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44cd83 (mulss 0.15)</t>
+        </is>
+      </c>
       <c r="M237" s="2" t="inlineStr"/>
       <c r="N237" s="2" t="inlineStr">
         <is>
@@ -11771,14 +12207,22 @@
       <c r="F239" s="2" t="inlineStr"/>
       <c r="G239" s="2" t="inlineStr">
         <is>
-          <t>Joint skill damage MegaUP</t>
+          <t>Joint skill damage +20%</t>
         </is>
       </c>
       <c r="H239" s="2" t="inlineStr"/>
-      <c r="I239" s="2" t="inlineStr"/>
+      <c r="I239" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J239" s="2" t="inlineStr"/>
       <c r="K239" s="2" t="inlineStr"/>
-      <c r="L239" s="2" t="inlineStr"/>
+      <c r="L239" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44c8ee (mulss 0.20)</t>
+        </is>
+      </c>
       <c r="M239" s="2" t="inlineStr"/>
       <c r="N239" s="2" t="inlineStr">
         <is>
@@ -11813,14 +12257,22 @@
       <c r="F240" s="2" t="inlineStr"/>
       <c r="G240" s="2" t="inlineStr">
         <is>
-          <t>Increase Mimic appearance rate in chests</t>
+          <t>Mimic chest rate +20%</t>
         </is>
       </c>
       <c r="H240" s="2" t="inlineStr"/>
-      <c r="I240" s="2" t="inlineStr"/>
+      <c r="I240" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J240" s="2" t="inlineStr"/>
       <c r="K240" s="2" t="inlineStr"/>
-      <c r="L240" s="2" t="inlineStr"/>
+      <c r="L240" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x55577a (+20% mimic chance)</t>
+        </is>
+      </c>
       <c r="M240" s="2" t="inlineStr"/>
       <c r="N240" s="2" t="inlineStr">
         <is>
@@ -12023,14 +12475,22 @@
       <c r="F245" s="2" t="inlineStr"/>
       <c r="G245" s="2" t="inlineStr">
         <is>
-          <t>May rarely recover all HP when turn starts</t>
+          <t>4% chance: full HP on turn</t>
         </is>
       </c>
       <c r="H245" s="2" t="inlineStr"/>
-      <c r="I245" s="2" t="inlineStr"/>
+      <c r="I245" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J245" s="2" t="inlineStr"/>
       <c r="K245" s="2" t="inlineStr"/>
-      <c r="L245" s="2" t="inlineStr"/>
+      <c r="L245" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x437d1a (4% full HP on turn)</t>
+        </is>
+      </c>
       <c r="M245" s="2" t="inlineStr"/>
       <c r="N245" s="2" t="inlineStr">
         <is>
@@ -12107,14 +12567,22 @@
       <c r="F247" s="2" t="inlineStr"/>
       <c r="G247" s="2" t="inlineStr">
         <is>
-          <t>Magic incantations go very fast... sometimes</t>
+          <t>Chant speed +25%</t>
         </is>
       </c>
       <c r="H247" s="2" t="inlineStr"/>
-      <c r="I247" s="2" t="inlineStr"/>
+      <c r="I247" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J247" s="2" t="inlineStr"/>
       <c r="K247" s="2" t="inlineStr"/>
-      <c r="L247" s="2" t="inlineStr"/>
+      <c r="L247" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44a380 (+25% chant speed)</t>
+        </is>
+      </c>
       <c r="M247" s="2" t="inlineStr"/>
       <c r="N247" s="2" t="inlineStr">
         <is>
@@ -12257,14 +12725,22 @@
       </c>
       <c r="G250" s="2" t="inlineStr">
         <is>
-          <t>Dance skill efficacy UP</t>
+          <t>Dance skill efficacy +2%</t>
         </is>
       </c>
       <c r="H250" s="2" t="inlineStr"/>
-      <c r="I250" s="2" t="inlineStr"/>
+      <c r="I250" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J250" s="2" t="inlineStr"/>
       <c r="K250" s="2" t="inlineStr"/>
-      <c r="L250" s="2" t="inlineStr"/>
+      <c r="L250" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x48c04a (mulss 0.02)</t>
+        </is>
+      </c>
       <c r="M250" s="2" t="inlineStr"/>
       <c r="N250" s="2" t="inlineStr">
         <is>
@@ -12299,14 +12775,22 @@
       <c r="F251" s="2" t="inlineStr"/>
       <c r="G251" s="2" t="inlineStr">
         <is>
-          <t>Dance skill efficacy UP</t>
+          <t>Dance skill efficacy +1%</t>
         </is>
       </c>
       <c r="H251" s="2" t="inlineStr"/>
-      <c r="I251" s="2" t="inlineStr"/>
+      <c r="I251" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J251" s="2" t="inlineStr"/>
       <c r="K251" s="2" t="inlineStr"/>
-      <c r="L251" s="2" t="inlineStr"/>
+      <c r="L251" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x48c07e (mulss 0.01)</t>
+        </is>
+      </c>
       <c r="M251" s="2" t="inlineStr"/>
       <c r="N251" s="2" t="inlineStr">
         <is>
@@ -12345,14 +12829,22 @@
       </c>
       <c r="G252" s="2" t="inlineStr">
         <is>
-          <t>Doll skill efficacy UP</t>
+          <t>Doll skill efficacy +2%</t>
         </is>
       </c>
       <c r="H252" s="2" t="inlineStr"/>
-      <c r="I252" s="2" t="inlineStr"/>
+      <c r="I252" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J252" s="2" t="inlineStr"/>
       <c r="K252" s="2" t="inlineStr"/>
-      <c r="L252" s="2" t="inlineStr"/>
+      <c r="L252" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44b533 (mulss 0.02)</t>
+        </is>
+      </c>
       <c r="M252" s="2" t="inlineStr"/>
       <c r="N252" s="2" t="inlineStr">
         <is>
@@ -12387,14 +12879,22 @@
       <c r="F253" s="2" t="inlineStr"/>
       <c r="G253" s="2" t="inlineStr">
         <is>
-          <t>Doll skill efficacy MiniUP</t>
+          <t>Doll skill efficacy +1%</t>
         </is>
       </c>
       <c r="H253" s="2" t="inlineStr"/>
-      <c r="I253" s="2" t="inlineStr"/>
+      <c r="I253" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
       <c r="J253" s="2" t="inlineStr"/>
       <c r="K253" s="2" t="inlineStr"/>
-      <c r="L253" s="2" t="inlineStr"/>
+      <c r="L253" s="2" t="inlineStr">
+        <is>
+          <t>x86: 0x44b58e (mulss 0.01)</t>
+        </is>
+      </c>
       <c r="M253" s="2" t="inlineStr"/>
       <c r="N253" s="2" t="inlineStr">
         <is>
@@ -13798,21 +14298,21 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>figure from dt2-wiki</t>
+          <t>figure from dt22-wiki</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>43</v>
+        <v>99</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>figure from dt22-wiki</t>
+          <t>figure from exe-verified</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="6">
@@ -13822,7 +14322,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>101</v>
+        <v>42</v>
       </c>
     </row>
   </sheetData>
@@ -13836,7 +14336,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="2" max="2"/>
@@ -13888,6 +14388,23 @@
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>exe-verified</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Directly decompiled from DT2-2 unwrapped x86 executable</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>yes</t>
         </is>

</xml_diff>